<commit_message>
Version 1.0.57 : catalogue par métier (10 activités, 691 produits, 9 rubriques) ; lecture du catalogue par pages ; modèles Excel par métier ; migration 20261018300000
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modeles/Mon-Dje-modele-produits.xlsx
+++ b/modeles/Mon-Dje-modele-produits.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mes produits" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemples" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listes" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemples" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4111,7 +4112,7 @@
       <formula2>80</formula2>
     </dataValidation>
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"pièce,bouteille,canette,casier,carton,sac,sachet,paquet,kg,litre,assiette,dose,tas,détail,demi,gros,article"</formula1>
+      <formula1>=Listes!$A$1:$A$38</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Prix de vente" error="Écrivez un nombre entier supérieur à 0, sans « F »." type="whole" errorStyle="warning" operator="greaterThanOrEqual">
       <formula1>1</formula1>
@@ -4135,6 +4136,287 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:A38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>pièce</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>bouteille</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>canette</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>casier</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>carton</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sac</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>sachet</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paquet</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>100 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10 g</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>litre</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>assiette</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>botte</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>détail</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>demi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>gros</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>boîte</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>pot</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>flacon</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>tube</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>bidon</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>seau</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>barre</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>rouleau</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>mètre</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>feuille</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>jeu</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>paire</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>balle</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ramette</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>plaque</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>part</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4387,7 +4669,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Version 1.0.64 : abonnement par le QR Wave de Mon Djê (paiement déclaré, confirmé par l'équipe), formules Petit/Moyen/Grand, pain manquant dans le stock et le résultat, prix de gros dans les modèles Excel, textes à lire vague 5 ; migrations 20261021300000 et 20261021400000
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modeles/Mon-Dje-modele-produits.xlsx
+++ b/modeles/Mon-Dje-modele-produits.xlsx
@@ -273,6 +273,11 @@
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>Facultatif. La quantité que vous avez aujourd’hui, en nombre entier. Si vide : 0.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Facultatif. Le prix quand vous livrez (au gros). Au comptoir, c’est toujours le prix de vente. Si vide : le prix de vente s’applique aux livraisons.</t>
       </text>
     </comment>
   </commentList>
@@ -568,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E501"/>
+  <dimension ref="A1:F501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -576,6 +581,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -602,6 +608,11 @@
       <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Stock</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Prix de gros</t>
         </is>
       </c>
     </row>
@@ -611,6 +622,7 @@
       <c r="C2" s="5" t="n"/>
       <c r="D2" s="5" t="n"/>
       <c r="E2" s="5" t="n"/>
+      <c r="F2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -618,6 +630,7 @@
       <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -625,6 +638,7 @@
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -632,6 +646,7 @@
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -639,6 +654,7 @@
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -646,6 +662,7 @@
       <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -653,6 +670,7 @@
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -660,6 +678,7 @@
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="n"/>
       <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -667,6 +686,7 @@
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="n"/>
       <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -674,6 +694,7 @@
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -681,6 +702,7 @@
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="n"/>
       <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -688,6 +710,7 @@
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="5" t="n"/>
       <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -695,6 +718,7 @@
       <c r="C14" s="5" t="n"/>
       <c r="D14" s="5" t="n"/>
       <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -702,6 +726,7 @@
       <c r="C15" s="5" t="n"/>
       <c r="D15" s="5" t="n"/>
       <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -709,6 +734,7 @@
       <c r="C16" s="5" t="n"/>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -716,6 +742,7 @@
       <c r="C17" s="5" t="n"/>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -723,6 +750,7 @@
       <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -730,6 +758,7 @@
       <c r="C19" s="5" t="n"/>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -737,6 +766,7 @@
       <c r="C20" s="5" t="n"/>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -744,6 +774,7 @@
       <c r="C21" s="5" t="n"/>
       <c r="D21" s="5" t="n"/>
       <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -751,6 +782,7 @@
       <c r="C22" s="5" t="n"/>
       <c r="D22" s="5" t="n"/>
       <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -758,6 +790,7 @@
       <c r="C23" s="5" t="n"/>
       <c r="D23" s="5" t="n"/>
       <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -765,6 +798,7 @@
       <c r="C24" s="5" t="n"/>
       <c r="D24" s="5" t="n"/>
       <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -772,6 +806,7 @@
       <c r="C25" s="5" t="n"/>
       <c r="D25" s="5" t="n"/>
       <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -779,6 +814,7 @@
       <c r="C26" s="5" t="n"/>
       <c r="D26" s="5" t="n"/>
       <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -786,6 +822,7 @@
       <c r="C27" s="5" t="n"/>
       <c r="D27" s="5" t="n"/>
       <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -793,6 +830,7 @@
       <c r="C28" s="5" t="n"/>
       <c r="D28" s="5" t="n"/>
       <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -800,6 +838,7 @@
       <c r="C29" s="5" t="n"/>
       <c r="D29" s="5" t="n"/>
       <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -807,6 +846,7 @@
       <c r="C30" s="5" t="n"/>
       <c r="D30" s="5" t="n"/>
       <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -814,6 +854,7 @@
       <c r="C31" s="5" t="n"/>
       <c r="D31" s="5" t="n"/>
       <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -821,6 +862,7 @@
       <c r="C32" s="5" t="n"/>
       <c r="D32" s="5" t="n"/>
       <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -828,6 +870,7 @@
       <c r="C33" s="5" t="n"/>
       <c r="D33" s="5" t="n"/>
       <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -835,6 +878,7 @@
       <c r="C34" s="5" t="n"/>
       <c r="D34" s="5" t="n"/>
       <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -842,6 +886,7 @@
       <c r="C35" s="5" t="n"/>
       <c r="D35" s="5" t="n"/>
       <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -849,6 +894,7 @@
       <c r="C36" s="5" t="n"/>
       <c r="D36" s="5" t="n"/>
       <c r="E36" s="5" t="n"/>
+      <c r="F36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -856,6 +902,7 @@
       <c r="C37" s="5" t="n"/>
       <c r="D37" s="5" t="n"/>
       <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -863,6 +910,7 @@
       <c r="C38" s="5" t="n"/>
       <c r="D38" s="5" t="n"/>
       <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -870,6 +918,7 @@
       <c r="C39" s="5" t="n"/>
       <c r="D39" s="5" t="n"/>
       <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -877,6 +926,7 @@
       <c r="C40" s="5" t="n"/>
       <c r="D40" s="5" t="n"/>
       <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -884,6 +934,7 @@
       <c r="C41" s="5" t="n"/>
       <c r="D41" s="5" t="n"/>
       <c r="E41" s="5" t="n"/>
+      <c r="F41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -891,6 +942,7 @@
       <c r="C42" s="5" t="n"/>
       <c r="D42" s="5" t="n"/>
       <c r="E42" s="5" t="n"/>
+      <c r="F42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -898,6 +950,7 @@
       <c r="C43" s="5" t="n"/>
       <c r="D43" s="5" t="n"/>
       <c r="E43" s="5" t="n"/>
+      <c r="F43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -905,6 +958,7 @@
       <c r="C44" s="5" t="n"/>
       <c r="D44" s="5" t="n"/>
       <c r="E44" s="5" t="n"/>
+      <c r="F44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -912,6 +966,7 @@
       <c r="C45" s="5" t="n"/>
       <c r="D45" s="5" t="n"/>
       <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -919,6 +974,7 @@
       <c r="C46" s="5" t="n"/>
       <c r="D46" s="5" t="n"/>
       <c r="E46" s="5" t="n"/>
+      <c r="F46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -926,6 +982,7 @@
       <c r="C47" s="5" t="n"/>
       <c r="D47" s="5" t="n"/>
       <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -933,6 +990,7 @@
       <c r="C48" s="5" t="n"/>
       <c r="D48" s="5" t="n"/>
       <c r="E48" s="5" t="n"/>
+      <c r="F48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -940,6 +998,7 @@
       <c r="C49" s="5" t="n"/>
       <c r="D49" s="5" t="n"/>
       <c r="E49" s="5" t="n"/>
+      <c r="F49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -947,6 +1006,7 @@
       <c r="C50" s="5" t="n"/>
       <c r="D50" s="5" t="n"/>
       <c r="E50" s="5" t="n"/>
+      <c r="F50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -954,6 +1014,7 @@
       <c r="C51" s="5" t="n"/>
       <c r="D51" s="5" t="n"/>
       <c r="E51" s="5" t="n"/>
+      <c r="F51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -961,6 +1022,7 @@
       <c r="C52" s="5" t="n"/>
       <c r="D52" s="5" t="n"/>
       <c r="E52" s="5" t="n"/>
+      <c r="F52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -968,6 +1030,7 @@
       <c r="C53" s="5" t="n"/>
       <c r="D53" s="5" t="n"/>
       <c r="E53" s="5" t="n"/>
+      <c r="F53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -975,6 +1038,7 @@
       <c r="C54" s="5" t="n"/>
       <c r="D54" s="5" t="n"/>
       <c r="E54" s="5" t="n"/>
+      <c r="F54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -982,6 +1046,7 @@
       <c r="C55" s="5" t="n"/>
       <c r="D55" s="5" t="n"/>
       <c r="E55" s="5" t="n"/>
+      <c r="F55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -989,6 +1054,7 @@
       <c r="C56" s="5" t="n"/>
       <c r="D56" s="5" t="n"/>
       <c r="E56" s="5" t="n"/>
+      <c r="F56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -996,6 +1062,7 @@
       <c r="C57" s="5" t="n"/>
       <c r="D57" s="5" t="n"/>
       <c r="E57" s="5" t="n"/>
+      <c r="F57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -1003,6 +1070,7 @@
       <c r="C58" s="5" t="n"/>
       <c r="D58" s="5" t="n"/>
       <c r="E58" s="5" t="n"/>
+      <c r="F58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -1010,6 +1078,7 @@
       <c r="C59" s="5" t="n"/>
       <c r="D59" s="5" t="n"/>
       <c r="E59" s="5" t="n"/>
+      <c r="F59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -1017,6 +1086,7 @@
       <c r="C60" s="5" t="n"/>
       <c r="D60" s="5" t="n"/>
       <c r="E60" s="5" t="n"/>
+      <c r="F60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -1024,6 +1094,7 @@
       <c r="C61" s="5" t="n"/>
       <c r="D61" s="5" t="n"/>
       <c r="E61" s="5" t="n"/>
+      <c r="F61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -1031,6 +1102,7 @@
       <c r="C62" s="5" t="n"/>
       <c r="D62" s="5" t="n"/>
       <c r="E62" s="5" t="n"/>
+      <c r="F62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
@@ -1038,6 +1110,7 @@
       <c r="C63" s="5" t="n"/>
       <c r="D63" s="5" t="n"/>
       <c r="E63" s="5" t="n"/>
+      <c r="F63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -1045,6 +1118,7 @@
       <c r="C64" s="5" t="n"/>
       <c r="D64" s="5" t="n"/>
       <c r="E64" s="5" t="n"/>
+      <c r="F64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -1052,6 +1126,7 @@
       <c r="C65" s="5" t="n"/>
       <c r="D65" s="5" t="n"/>
       <c r="E65" s="5" t="n"/>
+      <c r="F65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -1059,6 +1134,7 @@
       <c r="C66" s="5" t="n"/>
       <c r="D66" s="5" t="n"/>
       <c r="E66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -1066,6 +1142,7 @@
       <c r="C67" s="5" t="n"/>
       <c r="D67" s="5" t="n"/>
       <c r="E67" s="5" t="n"/>
+      <c r="F67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -1073,6 +1150,7 @@
       <c r="C68" s="5" t="n"/>
       <c r="D68" s="5" t="n"/>
       <c r="E68" s="5" t="n"/>
+      <c r="F68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
@@ -1080,6 +1158,7 @@
       <c r="C69" s="5" t="n"/>
       <c r="D69" s="5" t="n"/>
       <c r="E69" s="5" t="n"/>
+      <c r="F69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -1087,6 +1166,7 @@
       <c r="C70" s="5" t="n"/>
       <c r="D70" s="5" t="n"/>
       <c r="E70" s="5" t="n"/>
+      <c r="F70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
@@ -1094,6 +1174,7 @@
       <c r="C71" s="5" t="n"/>
       <c r="D71" s="5" t="n"/>
       <c r="E71" s="5" t="n"/>
+      <c r="F71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -1101,6 +1182,7 @@
       <c r="C72" s="5" t="n"/>
       <c r="D72" s="5" t="n"/>
       <c r="E72" s="5" t="n"/>
+      <c r="F72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
@@ -1108,6 +1190,7 @@
       <c r="C73" s="5" t="n"/>
       <c r="D73" s="5" t="n"/>
       <c r="E73" s="5" t="n"/>
+      <c r="F73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -1115,6 +1198,7 @@
       <c r="C74" s="5" t="n"/>
       <c r="D74" s="5" t="n"/>
       <c r="E74" s="5" t="n"/>
+      <c r="F74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
@@ -1122,6 +1206,7 @@
       <c r="C75" s="5" t="n"/>
       <c r="D75" s="5" t="n"/>
       <c r="E75" s="5" t="n"/>
+      <c r="F75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -1129,6 +1214,7 @@
       <c r="C76" s="5" t="n"/>
       <c r="D76" s="5" t="n"/>
       <c r="E76" s="5" t="n"/>
+      <c r="F76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -1136,6 +1222,7 @@
       <c r="C77" s="5" t="n"/>
       <c r="D77" s="5" t="n"/>
       <c r="E77" s="5" t="n"/>
+      <c r="F77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -1143,6 +1230,7 @@
       <c r="C78" s="5" t="n"/>
       <c r="D78" s="5" t="n"/>
       <c r="E78" s="5" t="n"/>
+      <c r="F78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
@@ -1150,6 +1238,7 @@
       <c r="C79" s="5" t="n"/>
       <c r="D79" s="5" t="n"/>
       <c r="E79" s="5" t="n"/>
+      <c r="F79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -1157,6 +1246,7 @@
       <c r="C80" s="5" t="n"/>
       <c r="D80" s="5" t="n"/>
       <c r="E80" s="5" t="n"/>
+      <c r="F80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
@@ -1164,6 +1254,7 @@
       <c r="C81" s="5" t="n"/>
       <c r="D81" s="5" t="n"/>
       <c r="E81" s="5" t="n"/>
+      <c r="F81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -1171,6 +1262,7 @@
       <c r="C82" s="5" t="n"/>
       <c r="D82" s="5" t="n"/>
       <c r="E82" s="5" t="n"/>
+      <c r="F82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n"/>
@@ -1178,6 +1270,7 @@
       <c r="C83" s="5" t="n"/>
       <c r="D83" s="5" t="n"/>
       <c r="E83" s="5" t="n"/>
+      <c r="F83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -1185,6 +1278,7 @@
       <c r="C84" s="5" t="n"/>
       <c r="D84" s="5" t="n"/>
       <c r="E84" s="5" t="n"/>
+      <c r="F84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n"/>
@@ -1192,6 +1286,7 @@
       <c r="C85" s="5" t="n"/>
       <c r="D85" s="5" t="n"/>
       <c r="E85" s="5" t="n"/>
+      <c r="F85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -1199,6 +1294,7 @@
       <c r="C86" s="5" t="n"/>
       <c r="D86" s="5" t="n"/>
       <c r="E86" s="5" t="n"/>
+      <c r="F86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n"/>
@@ -1206,6 +1302,7 @@
       <c r="C87" s="5" t="n"/>
       <c r="D87" s="5" t="n"/>
       <c r="E87" s="5" t="n"/>
+      <c r="F87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -1213,6 +1310,7 @@
       <c r="C88" s="5" t="n"/>
       <c r="D88" s="5" t="n"/>
       <c r="E88" s="5" t="n"/>
+      <c r="F88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n"/>
@@ -1220,6 +1318,7 @@
       <c r="C89" s="5" t="n"/>
       <c r="D89" s="5" t="n"/>
       <c r="E89" s="5" t="n"/>
+      <c r="F89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -1227,6 +1326,7 @@
       <c r="C90" s="5" t="n"/>
       <c r="D90" s="5" t="n"/>
       <c r="E90" s="5" t="n"/>
+      <c r="F90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n"/>
@@ -1234,6 +1334,7 @@
       <c r="C91" s="5" t="n"/>
       <c r="D91" s="5" t="n"/>
       <c r="E91" s="5" t="n"/>
+      <c r="F91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -1241,6 +1342,7 @@
       <c r="C92" s="5" t="n"/>
       <c r="D92" s="5" t="n"/>
       <c r="E92" s="5" t="n"/>
+      <c r="F92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n"/>
@@ -1248,6 +1350,7 @@
       <c r="C93" s="5" t="n"/>
       <c r="D93" s="5" t="n"/>
       <c r="E93" s="5" t="n"/>
+      <c r="F93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -1255,6 +1358,7 @@
       <c r="C94" s="5" t="n"/>
       <c r="D94" s="5" t="n"/>
       <c r="E94" s="5" t="n"/>
+      <c r="F94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n"/>
@@ -1262,6 +1366,7 @@
       <c r="C95" s="5" t="n"/>
       <c r="D95" s="5" t="n"/>
       <c r="E95" s="5" t="n"/>
+      <c r="F95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -1269,6 +1374,7 @@
       <c r="C96" s="5" t="n"/>
       <c r="D96" s="5" t="n"/>
       <c r="E96" s="5" t="n"/>
+      <c r="F96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n"/>
@@ -1276,6 +1382,7 @@
       <c r="C97" s="5" t="n"/>
       <c r="D97" s="5" t="n"/>
       <c r="E97" s="5" t="n"/>
+      <c r="F97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -1283,6 +1390,7 @@
       <c r="C98" s="5" t="n"/>
       <c r="D98" s="5" t="n"/>
       <c r="E98" s="5" t="n"/>
+      <c r="F98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n"/>
@@ -1290,6 +1398,7 @@
       <c r="C99" s="5" t="n"/>
       <c r="D99" s="5" t="n"/>
       <c r="E99" s="5" t="n"/>
+      <c r="F99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -1297,6 +1406,7 @@
       <c r="C100" s="5" t="n"/>
       <c r="D100" s="5" t="n"/>
       <c r="E100" s="5" t="n"/>
+      <c r="F100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n"/>
@@ -1304,6 +1414,7 @@
       <c r="C101" s="5" t="n"/>
       <c r="D101" s="5" t="n"/>
       <c r="E101" s="5" t="n"/>
+      <c r="F101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n"/>
@@ -1311,6 +1422,7 @@
       <c r="C102" s="5" t="n"/>
       <c r="D102" s="5" t="n"/>
       <c r="E102" s="5" t="n"/>
+      <c r="F102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n"/>
@@ -1318,6 +1430,7 @@
       <c r="C103" s="5" t="n"/>
       <c r="D103" s="5" t="n"/>
       <c r="E103" s="5" t="n"/>
+      <c r="F103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n"/>
@@ -1325,6 +1438,7 @@
       <c r="C104" s="5" t="n"/>
       <c r="D104" s="5" t="n"/>
       <c r="E104" s="5" t="n"/>
+      <c r="F104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n"/>
@@ -1332,6 +1446,7 @@
       <c r="C105" s="5" t="n"/>
       <c r="D105" s="5" t="n"/>
       <c r="E105" s="5" t="n"/>
+      <c r="F105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n"/>
@@ -1339,6 +1454,7 @@
       <c r="C106" s="5" t="n"/>
       <c r="D106" s="5" t="n"/>
       <c r="E106" s="5" t="n"/>
+      <c r="F106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n"/>
@@ -1346,6 +1462,7 @@
       <c r="C107" s="5" t="n"/>
       <c r="D107" s="5" t="n"/>
       <c r="E107" s="5" t="n"/>
+      <c r="F107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n"/>
@@ -1353,6 +1470,7 @@
       <c r="C108" s="5" t="n"/>
       <c r="D108" s="5" t="n"/>
       <c r="E108" s="5" t="n"/>
+      <c r="F108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n"/>
@@ -1360,6 +1478,7 @@
       <c r="C109" s="5" t="n"/>
       <c r="D109" s="5" t="n"/>
       <c r="E109" s="5" t="n"/>
+      <c r="F109" s="5" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n"/>
@@ -1367,6 +1486,7 @@
       <c r="C110" s="5" t="n"/>
       <c r="D110" s="5" t="n"/>
       <c r="E110" s="5" t="n"/>
+      <c r="F110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n"/>
@@ -1374,6 +1494,7 @@
       <c r="C111" s="5" t="n"/>
       <c r="D111" s="5" t="n"/>
       <c r="E111" s="5" t="n"/>
+      <c r="F111" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="3" t="n"/>
@@ -1381,6 +1502,7 @@
       <c r="C112" s="5" t="n"/>
       <c r="D112" s="5" t="n"/>
       <c r="E112" s="5" t="n"/>
+      <c r="F112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n"/>
@@ -1388,6 +1510,7 @@
       <c r="C113" s="5" t="n"/>
       <c r="D113" s="5" t="n"/>
       <c r="E113" s="5" t="n"/>
+      <c r="F113" s="5" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n"/>
@@ -1395,6 +1518,7 @@
       <c r="C114" s="5" t="n"/>
       <c r="D114" s="5" t="n"/>
       <c r="E114" s="5" t="n"/>
+      <c r="F114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n"/>
@@ -1402,6 +1526,7 @@
       <c r="C115" s="5" t="n"/>
       <c r="D115" s="5" t="n"/>
       <c r="E115" s="5" t="n"/>
+      <c r="F115" s="5" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n"/>
@@ -1409,6 +1534,7 @@
       <c r="C116" s="5" t="n"/>
       <c r="D116" s="5" t="n"/>
       <c r="E116" s="5" t="n"/>
+      <c r="F116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="3" t="n"/>
@@ -1416,6 +1542,7 @@
       <c r="C117" s="5" t="n"/>
       <c r="D117" s="5" t="n"/>
       <c r="E117" s="5" t="n"/>
+      <c r="F117" s="5" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n"/>
@@ -1423,6 +1550,7 @@
       <c r="C118" s="5" t="n"/>
       <c r="D118" s="5" t="n"/>
       <c r="E118" s="5" t="n"/>
+      <c r="F118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="n"/>
@@ -1430,6 +1558,7 @@
       <c r="C119" s="5" t="n"/>
       <c r="D119" s="5" t="n"/>
       <c r="E119" s="5" t="n"/>
+      <c r="F119" s="5" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="n"/>
@@ -1437,6 +1566,7 @@
       <c r="C120" s="5" t="n"/>
       <c r="D120" s="5" t="n"/>
       <c r="E120" s="5" t="n"/>
+      <c r="F120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="n"/>
@@ -1444,6 +1574,7 @@
       <c r="C121" s="5" t="n"/>
       <c r="D121" s="5" t="n"/>
       <c r="E121" s="5" t="n"/>
+      <c r="F121" s="5" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n"/>
@@ -1451,6 +1582,7 @@
       <c r="C122" s="5" t="n"/>
       <c r="D122" s="5" t="n"/>
       <c r="E122" s="5" t="n"/>
+      <c r="F122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="n"/>
@@ -1458,6 +1590,7 @@
       <c r="C123" s="5" t="n"/>
       <c r="D123" s="5" t="n"/>
       <c r="E123" s="5" t="n"/>
+      <c r="F123" s="5" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n"/>
@@ -1465,6 +1598,7 @@
       <c r="C124" s="5" t="n"/>
       <c r="D124" s="5" t="n"/>
       <c r="E124" s="5" t="n"/>
+      <c r="F124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n"/>
@@ -1472,6 +1606,7 @@
       <c r="C125" s="5" t="n"/>
       <c r="D125" s="5" t="n"/>
       <c r="E125" s="5" t="n"/>
+      <c r="F125" s="5" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n"/>
@@ -1479,6 +1614,7 @@
       <c r="C126" s="5" t="n"/>
       <c r="D126" s="5" t="n"/>
       <c r="E126" s="5" t="n"/>
+      <c r="F126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="3" t="n"/>
@@ -1486,6 +1622,7 @@
       <c r="C127" s="5" t="n"/>
       <c r="D127" s="5" t="n"/>
       <c r="E127" s="5" t="n"/>
+      <c r="F127" s="5" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="n"/>
@@ -1493,6 +1630,7 @@
       <c r="C128" s="5" t="n"/>
       <c r="D128" s="5" t="n"/>
       <c r="E128" s="5" t="n"/>
+      <c r="F128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="3" t="n"/>
@@ -1500,6 +1638,7 @@
       <c r="C129" s="5" t="n"/>
       <c r="D129" s="5" t="n"/>
       <c r="E129" s="5" t="n"/>
+      <c r="F129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n"/>
@@ -1507,6 +1646,7 @@
       <c r="C130" s="5" t="n"/>
       <c r="D130" s="5" t="n"/>
       <c r="E130" s="5" t="n"/>
+      <c r="F130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="n"/>
@@ -1514,6 +1654,7 @@
       <c r="C131" s="5" t="n"/>
       <c r="D131" s="5" t="n"/>
       <c r="E131" s="5" t="n"/>
+      <c r="F131" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n"/>
@@ -1521,6 +1662,7 @@
       <c r="C132" s="5" t="n"/>
       <c r="D132" s="5" t="n"/>
       <c r="E132" s="5" t="n"/>
+      <c r="F132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="3" t="n"/>
@@ -1528,6 +1670,7 @@
       <c r="C133" s="5" t="n"/>
       <c r="D133" s="5" t="n"/>
       <c r="E133" s="5" t="n"/>
+      <c r="F133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="3" t="n"/>
@@ -1535,6 +1678,7 @@
       <c r="C134" s="5" t="n"/>
       <c r="D134" s="5" t="n"/>
       <c r="E134" s="5" t="n"/>
+      <c r="F134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="3" t="n"/>
@@ -1542,6 +1686,7 @@
       <c r="C135" s="5" t="n"/>
       <c r="D135" s="5" t="n"/>
       <c r="E135" s="5" t="n"/>
+      <c r="F135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="n"/>
@@ -1549,6 +1694,7 @@
       <c r="C136" s="5" t="n"/>
       <c r="D136" s="5" t="n"/>
       <c r="E136" s="5" t="n"/>
+      <c r="F136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="3" t="n"/>
@@ -1556,6 +1702,7 @@
       <c r="C137" s="5" t="n"/>
       <c r="D137" s="5" t="n"/>
       <c r="E137" s="5" t="n"/>
+      <c r="F137" s="5" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="3" t="n"/>
@@ -1563,6 +1710,7 @@
       <c r="C138" s="5" t="n"/>
       <c r="D138" s="5" t="n"/>
       <c r="E138" s="5" t="n"/>
+      <c r="F138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="3" t="n"/>
@@ -1570,6 +1718,7 @@
       <c r="C139" s="5" t="n"/>
       <c r="D139" s="5" t="n"/>
       <c r="E139" s="5" t="n"/>
+      <c r="F139" s="5" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n"/>
@@ -1577,6 +1726,7 @@
       <c r="C140" s="5" t="n"/>
       <c r="D140" s="5" t="n"/>
       <c r="E140" s="5" t="n"/>
+      <c r="F140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="3" t="n"/>
@@ -1584,6 +1734,7 @@
       <c r="C141" s="5" t="n"/>
       <c r="D141" s="5" t="n"/>
       <c r="E141" s="5" t="n"/>
+      <c r="F141" s="5" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="3" t="n"/>
@@ -1591,6 +1742,7 @@
       <c r="C142" s="5" t="n"/>
       <c r="D142" s="5" t="n"/>
       <c r="E142" s="5" t="n"/>
+      <c r="F142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="3" t="n"/>
@@ -1598,6 +1750,7 @@
       <c r="C143" s="5" t="n"/>
       <c r="D143" s="5" t="n"/>
       <c r="E143" s="5" t="n"/>
+      <c r="F143" s="5" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="3" t="n"/>
@@ -1605,6 +1758,7 @@
       <c r="C144" s="5" t="n"/>
       <c r="D144" s="5" t="n"/>
       <c r="E144" s="5" t="n"/>
+      <c r="F144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="3" t="n"/>
@@ -1612,6 +1766,7 @@
       <c r="C145" s="5" t="n"/>
       <c r="D145" s="5" t="n"/>
       <c r="E145" s="5" t="n"/>
+      <c r="F145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="3" t="n"/>
@@ -1619,6 +1774,7 @@
       <c r="C146" s="5" t="n"/>
       <c r="D146" s="5" t="n"/>
       <c r="E146" s="5" t="n"/>
+      <c r="F146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="n"/>
@@ -1626,6 +1782,7 @@
       <c r="C147" s="5" t="n"/>
       <c r="D147" s="5" t="n"/>
       <c r="E147" s="5" t="n"/>
+      <c r="F147" s="5" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="3" t="n"/>
@@ -1633,6 +1790,7 @@
       <c r="C148" s="5" t="n"/>
       <c r="D148" s="5" t="n"/>
       <c r="E148" s="5" t="n"/>
+      <c r="F148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="3" t="n"/>
@@ -1640,6 +1798,7 @@
       <c r="C149" s="5" t="n"/>
       <c r="D149" s="5" t="n"/>
       <c r="E149" s="5" t="n"/>
+      <c r="F149" s="5" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="3" t="n"/>
@@ -1647,6 +1806,7 @@
       <c r="C150" s="5" t="n"/>
       <c r="D150" s="5" t="n"/>
       <c r="E150" s="5" t="n"/>
+      <c r="F150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="3" t="n"/>
@@ -1654,6 +1814,7 @@
       <c r="C151" s="5" t="n"/>
       <c r="D151" s="5" t="n"/>
       <c r="E151" s="5" t="n"/>
+      <c r="F151" s="5" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="3" t="n"/>
@@ -1661,6 +1822,7 @@
       <c r="C152" s="5" t="n"/>
       <c r="D152" s="5" t="n"/>
       <c r="E152" s="5" t="n"/>
+      <c r="F152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="n"/>
@@ -1668,6 +1830,7 @@
       <c r="C153" s="5" t="n"/>
       <c r="D153" s="5" t="n"/>
       <c r="E153" s="5" t="n"/>
+      <c r="F153" s="5" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="n"/>
@@ -1675,6 +1838,7 @@
       <c r="C154" s="5" t="n"/>
       <c r="D154" s="5" t="n"/>
       <c r="E154" s="5" t="n"/>
+      <c r="F154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="3" t="n"/>
@@ -1682,6 +1846,7 @@
       <c r="C155" s="5" t="n"/>
       <c r="D155" s="5" t="n"/>
       <c r="E155" s="5" t="n"/>
+      <c r="F155" s="5" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="n"/>
@@ -1689,6 +1854,7 @@
       <c r="C156" s="5" t="n"/>
       <c r="D156" s="5" t="n"/>
       <c r="E156" s="5" t="n"/>
+      <c r="F156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="3" t="n"/>
@@ -1696,6 +1862,7 @@
       <c r="C157" s="5" t="n"/>
       <c r="D157" s="5" t="n"/>
       <c r="E157" s="5" t="n"/>
+      <c r="F157" s="5" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="3" t="n"/>
@@ -1703,6 +1870,7 @@
       <c r="C158" s="5" t="n"/>
       <c r="D158" s="5" t="n"/>
       <c r="E158" s="5" t="n"/>
+      <c r="F158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="3" t="n"/>
@@ -1710,6 +1878,7 @@
       <c r="C159" s="5" t="n"/>
       <c r="D159" s="5" t="n"/>
       <c r="E159" s="5" t="n"/>
+      <c r="F159" s="5" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="3" t="n"/>
@@ -1717,6 +1886,7 @@
       <c r="C160" s="5" t="n"/>
       <c r="D160" s="5" t="n"/>
       <c r="E160" s="5" t="n"/>
+      <c r="F160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="3" t="n"/>
@@ -1724,6 +1894,7 @@
       <c r="C161" s="5" t="n"/>
       <c r="D161" s="5" t="n"/>
       <c r="E161" s="5" t="n"/>
+      <c r="F161" s="5" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="3" t="n"/>
@@ -1731,6 +1902,7 @@
       <c r="C162" s="5" t="n"/>
       <c r="D162" s="5" t="n"/>
       <c r="E162" s="5" t="n"/>
+      <c r="F162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="3" t="n"/>
@@ -1738,6 +1910,7 @@
       <c r="C163" s="5" t="n"/>
       <c r="D163" s="5" t="n"/>
       <c r="E163" s="5" t="n"/>
+      <c r="F163" s="5" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="3" t="n"/>
@@ -1745,6 +1918,7 @@
       <c r="C164" s="5" t="n"/>
       <c r="D164" s="5" t="n"/>
       <c r="E164" s="5" t="n"/>
+      <c r="F164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="3" t="n"/>
@@ -1752,6 +1926,7 @@
       <c r="C165" s="5" t="n"/>
       <c r="D165" s="5" t="n"/>
       <c r="E165" s="5" t="n"/>
+      <c r="F165" s="5" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="3" t="n"/>
@@ -1759,6 +1934,7 @@
       <c r="C166" s="5" t="n"/>
       <c r="D166" s="5" t="n"/>
       <c r="E166" s="5" t="n"/>
+      <c r="F166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="3" t="n"/>
@@ -1766,6 +1942,7 @@
       <c r="C167" s="5" t="n"/>
       <c r="D167" s="5" t="n"/>
       <c r="E167" s="5" t="n"/>
+      <c r="F167" s="5" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="3" t="n"/>
@@ -1773,6 +1950,7 @@
       <c r="C168" s="5" t="n"/>
       <c r="D168" s="5" t="n"/>
       <c r="E168" s="5" t="n"/>
+      <c r="F168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="3" t="n"/>
@@ -1780,6 +1958,7 @@
       <c r="C169" s="5" t="n"/>
       <c r="D169" s="5" t="n"/>
       <c r="E169" s="5" t="n"/>
+      <c r="F169" s="5" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="n"/>
@@ -1787,6 +1966,7 @@
       <c r="C170" s="5" t="n"/>
       <c r="D170" s="5" t="n"/>
       <c r="E170" s="5" t="n"/>
+      <c r="F170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="3" t="n"/>
@@ -1794,6 +1974,7 @@
       <c r="C171" s="5" t="n"/>
       <c r="D171" s="5" t="n"/>
       <c r="E171" s="5" t="n"/>
+      <c r="F171" s="5" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="3" t="n"/>
@@ -1801,6 +1982,7 @@
       <c r="C172" s="5" t="n"/>
       <c r="D172" s="5" t="n"/>
       <c r="E172" s="5" t="n"/>
+      <c r="F172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="3" t="n"/>
@@ -1808,6 +1990,7 @@
       <c r="C173" s="5" t="n"/>
       <c r="D173" s="5" t="n"/>
       <c r="E173" s="5" t="n"/>
+      <c r="F173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="3" t="n"/>
@@ -1815,6 +1998,7 @@
       <c r="C174" s="5" t="n"/>
       <c r="D174" s="5" t="n"/>
       <c r="E174" s="5" t="n"/>
+      <c r="F174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="3" t="n"/>
@@ -1822,6 +2006,7 @@
       <c r="C175" s="5" t="n"/>
       <c r="D175" s="5" t="n"/>
       <c r="E175" s="5" t="n"/>
+      <c r="F175" s="5" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="3" t="n"/>
@@ -1829,6 +2014,7 @@
       <c r="C176" s="5" t="n"/>
       <c r="D176" s="5" t="n"/>
       <c r="E176" s="5" t="n"/>
+      <c r="F176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="3" t="n"/>
@@ -1836,6 +2022,7 @@
       <c r="C177" s="5" t="n"/>
       <c r="D177" s="5" t="n"/>
       <c r="E177" s="5" t="n"/>
+      <c r="F177" s="5" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="n"/>
@@ -1843,6 +2030,7 @@
       <c r="C178" s="5" t="n"/>
       <c r="D178" s="5" t="n"/>
       <c r="E178" s="5" t="n"/>
+      <c r="F178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="3" t="n"/>
@@ -1850,6 +2038,7 @@
       <c r="C179" s="5" t="n"/>
       <c r="D179" s="5" t="n"/>
       <c r="E179" s="5" t="n"/>
+      <c r="F179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="3" t="n"/>
@@ -1857,6 +2046,7 @@
       <c r="C180" s="5" t="n"/>
       <c r="D180" s="5" t="n"/>
       <c r="E180" s="5" t="n"/>
+      <c r="F180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="3" t="n"/>
@@ -1864,6 +2054,7 @@
       <c r="C181" s="5" t="n"/>
       <c r="D181" s="5" t="n"/>
       <c r="E181" s="5" t="n"/>
+      <c r="F181" s="5" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="3" t="n"/>
@@ -1871,6 +2062,7 @@
       <c r="C182" s="5" t="n"/>
       <c r="D182" s="5" t="n"/>
       <c r="E182" s="5" t="n"/>
+      <c r="F182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="n"/>
@@ -1878,6 +2070,7 @@
       <c r="C183" s="5" t="n"/>
       <c r="D183" s="5" t="n"/>
       <c r="E183" s="5" t="n"/>
+      <c r="F183" s="5" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="n"/>
@@ -1885,6 +2078,7 @@
       <c r="C184" s="5" t="n"/>
       <c r="D184" s="5" t="n"/>
       <c r="E184" s="5" t="n"/>
+      <c r="F184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="n"/>
@@ -1892,6 +2086,7 @@
       <c r="C185" s="5" t="n"/>
       <c r="D185" s="5" t="n"/>
       <c r="E185" s="5" t="n"/>
+      <c r="F185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="3" t="n"/>
@@ -1899,6 +2094,7 @@
       <c r="C186" s="5" t="n"/>
       <c r="D186" s="5" t="n"/>
       <c r="E186" s="5" t="n"/>
+      <c r="F186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="n"/>
@@ -1906,6 +2102,7 @@
       <c r="C187" s="5" t="n"/>
       <c r="D187" s="5" t="n"/>
       <c r="E187" s="5" t="n"/>
+      <c r="F187" s="5" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="3" t="n"/>
@@ -1913,6 +2110,7 @@
       <c r="C188" s="5" t="n"/>
       <c r="D188" s="5" t="n"/>
       <c r="E188" s="5" t="n"/>
+      <c r="F188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="3" t="n"/>
@@ -1920,6 +2118,7 @@
       <c r="C189" s="5" t="n"/>
       <c r="D189" s="5" t="n"/>
       <c r="E189" s="5" t="n"/>
+      <c r="F189" s="5" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="3" t="n"/>
@@ -1927,6 +2126,7 @@
       <c r="C190" s="5" t="n"/>
       <c r="D190" s="5" t="n"/>
       <c r="E190" s="5" t="n"/>
+      <c r="F190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="3" t="n"/>
@@ -1934,6 +2134,7 @@
       <c r="C191" s="5" t="n"/>
       <c r="D191" s="5" t="n"/>
       <c r="E191" s="5" t="n"/>
+      <c r="F191" s="5" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n"/>
@@ -1941,6 +2142,7 @@
       <c r="C192" s="5" t="n"/>
       <c r="D192" s="5" t="n"/>
       <c r="E192" s="5" t="n"/>
+      <c r="F192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="3" t="n"/>
@@ -1948,6 +2150,7 @@
       <c r="C193" s="5" t="n"/>
       <c r="D193" s="5" t="n"/>
       <c r="E193" s="5" t="n"/>
+      <c r="F193" s="5" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="3" t="n"/>
@@ -1955,6 +2158,7 @@
       <c r="C194" s="5" t="n"/>
       <c r="D194" s="5" t="n"/>
       <c r="E194" s="5" t="n"/>
+      <c r="F194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="3" t="n"/>
@@ -1962,6 +2166,7 @@
       <c r="C195" s="5" t="n"/>
       <c r="D195" s="5" t="n"/>
       <c r="E195" s="5" t="n"/>
+      <c r="F195" s="5" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="3" t="n"/>
@@ -1969,6 +2174,7 @@
       <c r="C196" s="5" t="n"/>
       <c r="D196" s="5" t="n"/>
       <c r="E196" s="5" t="n"/>
+      <c r="F196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="3" t="n"/>
@@ -1976,6 +2182,7 @@
       <c r="C197" s="5" t="n"/>
       <c r="D197" s="5" t="n"/>
       <c r="E197" s="5" t="n"/>
+      <c r="F197" s="5" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="3" t="n"/>
@@ -1983,6 +2190,7 @@
       <c r="C198" s="5" t="n"/>
       <c r="D198" s="5" t="n"/>
       <c r="E198" s="5" t="n"/>
+      <c r="F198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="3" t="n"/>
@@ -1990,6 +2198,7 @@
       <c r="C199" s="5" t="n"/>
       <c r="D199" s="5" t="n"/>
       <c r="E199" s="5" t="n"/>
+      <c r="F199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="3" t="n"/>
@@ -1997,6 +2206,7 @@
       <c r="C200" s="5" t="n"/>
       <c r="D200" s="5" t="n"/>
       <c r="E200" s="5" t="n"/>
+      <c r="F200" s="5" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="3" t="n"/>
@@ -2004,6 +2214,7 @@
       <c r="C201" s="5" t="n"/>
       <c r="D201" s="5" t="n"/>
       <c r="E201" s="5" t="n"/>
+      <c r="F201" s="5" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="3" t="n"/>
@@ -2011,6 +2222,7 @@
       <c r="C202" s="5" t="n"/>
       <c r="D202" s="5" t="n"/>
       <c r="E202" s="5" t="n"/>
+      <c r="F202" s="5" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="3" t="n"/>
@@ -2018,6 +2230,7 @@
       <c r="C203" s="5" t="n"/>
       <c r="D203" s="5" t="n"/>
       <c r="E203" s="5" t="n"/>
+      <c r="F203" s="5" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="3" t="n"/>
@@ -2025,6 +2238,7 @@
       <c r="C204" s="5" t="n"/>
       <c r="D204" s="5" t="n"/>
       <c r="E204" s="5" t="n"/>
+      <c r="F204" s="5" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="3" t="n"/>
@@ -2032,6 +2246,7 @@
       <c r="C205" s="5" t="n"/>
       <c r="D205" s="5" t="n"/>
       <c r="E205" s="5" t="n"/>
+      <c r="F205" s="5" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="3" t="n"/>
@@ -2039,6 +2254,7 @@
       <c r="C206" s="5" t="n"/>
       <c r="D206" s="5" t="n"/>
       <c r="E206" s="5" t="n"/>
+      <c r="F206" s="5" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="3" t="n"/>
@@ -2046,6 +2262,7 @@
       <c r="C207" s="5" t="n"/>
       <c r="D207" s="5" t="n"/>
       <c r="E207" s="5" t="n"/>
+      <c r="F207" s="5" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="3" t="n"/>
@@ -2053,6 +2270,7 @@
       <c r="C208" s="5" t="n"/>
       <c r="D208" s="5" t="n"/>
       <c r="E208" s="5" t="n"/>
+      <c r="F208" s="5" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="3" t="n"/>
@@ -2060,6 +2278,7 @@
       <c r="C209" s="5" t="n"/>
       <c r="D209" s="5" t="n"/>
       <c r="E209" s="5" t="n"/>
+      <c r="F209" s="5" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="3" t="n"/>
@@ -2067,6 +2286,7 @@
       <c r="C210" s="5" t="n"/>
       <c r="D210" s="5" t="n"/>
       <c r="E210" s="5" t="n"/>
+      <c r="F210" s="5" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="3" t="n"/>
@@ -2074,6 +2294,7 @@
       <c r="C211" s="5" t="n"/>
       <c r="D211" s="5" t="n"/>
       <c r="E211" s="5" t="n"/>
+      <c r="F211" s="5" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="3" t="n"/>
@@ -2081,6 +2302,7 @@
       <c r="C212" s="5" t="n"/>
       <c r="D212" s="5" t="n"/>
       <c r="E212" s="5" t="n"/>
+      <c r="F212" s="5" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="3" t="n"/>
@@ -2088,6 +2310,7 @@
       <c r="C213" s="5" t="n"/>
       <c r="D213" s="5" t="n"/>
       <c r="E213" s="5" t="n"/>
+      <c r="F213" s="5" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="3" t="n"/>
@@ -2095,6 +2318,7 @@
       <c r="C214" s="5" t="n"/>
       <c r="D214" s="5" t="n"/>
       <c r="E214" s="5" t="n"/>
+      <c r="F214" s="5" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="3" t="n"/>
@@ -2102,6 +2326,7 @@
       <c r="C215" s="5" t="n"/>
       <c r="D215" s="5" t="n"/>
       <c r="E215" s="5" t="n"/>
+      <c r="F215" s="5" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="3" t="n"/>
@@ -2109,6 +2334,7 @@
       <c r="C216" s="5" t="n"/>
       <c r="D216" s="5" t="n"/>
       <c r="E216" s="5" t="n"/>
+      <c r="F216" s="5" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="3" t="n"/>
@@ -2116,6 +2342,7 @@
       <c r="C217" s="5" t="n"/>
       <c r="D217" s="5" t="n"/>
       <c r="E217" s="5" t="n"/>
+      <c r="F217" s="5" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="3" t="n"/>
@@ -2123,6 +2350,7 @@
       <c r="C218" s="5" t="n"/>
       <c r="D218" s="5" t="n"/>
       <c r="E218" s="5" t="n"/>
+      <c r="F218" s="5" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="3" t="n"/>
@@ -2130,6 +2358,7 @@
       <c r="C219" s="5" t="n"/>
       <c r="D219" s="5" t="n"/>
       <c r="E219" s="5" t="n"/>
+      <c r="F219" s="5" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="3" t="n"/>
@@ -2137,6 +2366,7 @@
       <c r="C220" s="5" t="n"/>
       <c r="D220" s="5" t="n"/>
       <c r="E220" s="5" t="n"/>
+      <c r="F220" s="5" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="3" t="n"/>
@@ -2144,6 +2374,7 @@
       <c r="C221" s="5" t="n"/>
       <c r="D221" s="5" t="n"/>
       <c r="E221" s="5" t="n"/>
+      <c r="F221" s="5" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="3" t="n"/>
@@ -2151,6 +2382,7 @@
       <c r="C222" s="5" t="n"/>
       <c r="D222" s="5" t="n"/>
       <c r="E222" s="5" t="n"/>
+      <c r="F222" s="5" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="3" t="n"/>
@@ -2158,6 +2390,7 @@
       <c r="C223" s="5" t="n"/>
       <c r="D223" s="5" t="n"/>
       <c r="E223" s="5" t="n"/>
+      <c r="F223" s="5" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="3" t="n"/>
@@ -2165,6 +2398,7 @@
       <c r="C224" s="5" t="n"/>
       <c r="D224" s="5" t="n"/>
       <c r="E224" s="5" t="n"/>
+      <c r="F224" s="5" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="3" t="n"/>
@@ -2172,6 +2406,7 @@
       <c r="C225" s="5" t="n"/>
       <c r="D225" s="5" t="n"/>
       <c r="E225" s="5" t="n"/>
+      <c r="F225" s="5" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="3" t="n"/>
@@ -2179,6 +2414,7 @@
       <c r="C226" s="5" t="n"/>
       <c r="D226" s="5" t="n"/>
       <c r="E226" s="5" t="n"/>
+      <c r="F226" s="5" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="3" t="n"/>
@@ -2186,6 +2422,7 @@
       <c r="C227" s="5" t="n"/>
       <c r="D227" s="5" t="n"/>
       <c r="E227" s="5" t="n"/>
+      <c r="F227" s="5" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="3" t="n"/>
@@ -2193,6 +2430,7 @@
       <c r="C228" s="5" t="n"/>
       <c r="D228" s="5" t="n"/>
       <c r="E228" s="5" t="n"/>
+      <c r="F228" s="5" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="3" t="n"/>
@@ -2200,6 +2438,7 @@
       <c r="C229" s="5" t="n"/>
       <c r="D229" s="5" t="n"/>
       <c r="E229" s="5" t="n"/>
+      <c r="F229" s="5" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="3" t="n"/>
@@ -2207,6 +2446,7 @@
       <c r="C230" s="5" t="n"/>
       <c r="D230" s="5" t="n"/>
       <c r="E230" s="5" t="n"/>
+      <c r="F230" s="5" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="3" t="n"/>
@@ -2214,6 +2454,7 @@
       <c r="C231" s="5" t="n"/>
       <c r="D231" s="5" t="n"/>
       <c r="E231" s="5" t="n"/>
+      <c r="F231" s="5" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="3" t="n"/>
@@ -2221,6 +2462,7 @@
       <c r="C232" s="5" t="n"/>
       <c r="D232" s="5" t="n"/>
       <c r="E232" s="5" t="n"/>
+      <c r="F232" s="5" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="3" t="n"/>
@@ -2228,6 +2470,7 @@
       <c r="C233" s="5" t="n"/>
       <c r="D233" s="5" t="n"/>
       <c r="E233" s="5" t="n"/>
+      <c r="F233" s="5" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="3" t="n"/>
@@ -2235,6 +2478,7 @@
       <c r="C234" s="5" t="n"/>
       <c r="D234" s="5" t="n"/>
       <c r="E234" s="5" t="n"/>
+      <c r="F234" s="5" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="3" t="n"/>
@@ -2242,6 +2486,7 @@
       <c r="C235" s="5" t="n"/>
       <c r="D235" s="5" t="n"/>
       <c r="E235" s="5" t="n"/>
+      <c r="F235" s="5" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="3" t="n"/>
@@ -2249,6 +2494,7 @@
       <c r="C236" s="5" t="n"/>
       <c r="D236" s="5" t="n"/>
       <c r="E236" s="5" t="n"/>
+      <c r="F236" s="5" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="3" t="n"/>
@@ -2256,6 +2502,7 @@
       <c r="C237" s="5" t="n"/>
       <c r="D237" s="5" t="n"/>
       <c r="E237" s="5" t="n"/>
+      <c r="F237" s="5" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="3" t="n"/>
@@ -2263,6 +2510,7 @@
       <c r="C238" s="5" t="n"/>
       <c r="D238" s="5" t="n"/>
       <c r="E238" s="5" t="n"/>
+      <c r="F238" s="5" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="3" t="n"/>
@@ -2270,6 +2518,7 @@
       <c r="C239" s="5" t="n"/>
       <c r="D239" s="5" t="n"/>
       <c r="E239" s="5" t="n"/>
+      <c r="F239" s="5" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="3" t="n"/>
@@ -2277,6 +2526,7 @@
       <c r="C240" s="5" t="n"/>
       <c r="D240" s="5" t="n"/>
       <c r="E240" s="5" t="n"/>
+      <c r="F240" s="5" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="3" t="n"/>
@@ -2284,6 +2534,7 @@
       <c r="C241" s="5" t="n"/>
       <c r="D241" s="5" t="n"/>
       <c r="E241" s="5" t="n"/>
+      <c r="F241" s="5" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="3" t="n"/>
@@ -2291,6 +2542,7 @@
       <c r="C242" s="5" t="n"/>
       <c r="D242" s="5" t="n"/>
       <c r="E242" s="5" t="n"/>
+      <c r="F242" s="5" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="3" t="n"/>
@@ -2298,6 +2550,7 @@
       <c r="C243" s="5" t="n"/>
       <c r="D243" s="5" t="n"/>
       <c r="E243" s="5" t="n"/>
+      <c r="F243" s="5" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="3" t="n"/>
@@ -2305,6 +2558,7 @@
       <c r="C244" s="5" t="n"/>
       <c r="D244" s="5" t="n"/>
       <c r="E244" s="5" t="n"/>
+      <c r="F244" s="5" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="3" t="n"/>
@@ -2312,6 +2566,7 @@
       <c r="C245" s="5" t="n"/>
       <c r="D245" s="5" t="n"/>
       <c r="E245" s="5" t="n"/>
+      <c r="F245" s="5" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="3" t="n"/>
@@ -2319,6 +2574,7 @@
       <c r="C246" s="5" t="n"/>
       <c r="D246" s="5" t="n"/>
       <c r="E246" s="5" t="n"/>
+      <c r="F246" s="5" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="3" t="n"/>
@@ -2326,6 +2582,7 @@
       <c r="C247" s="5" t="n"/>
       <c r="D247" s="5" t="n"/>
       <c r="E247" s="5" t="n"/>
+      <c r="F247" s="5" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="3" t="n"/>
@@ -2333,6 +2590,7 @@
       <c r="C248" s="5" t="n"/>
       <c r="D248" s="5" t="n"/>
       <c r="E248" s="5" t="n"/>
+      <c r="F248" s="5" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="3" t="n"/>
@@ -2340,6 +2598,7 @@
       <c r="C249" s="5" t="n"/>
       <c r="D249" s="5" t="n"/>
       <c r="E249" s="5" t="n"/>
+      <c r="F249" s="5" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="3" t="n"/>
@@ -2347,6 +2606,7 @@
       <c r="C250" s="5" t="n"/>
       <c r="D250" s="5" t="n"/>
       <c r="E250" s="5" t="n"/>
+      <c r="F250" s="5" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="3" t="n"/>
@@ -2354,6 +2614,7 @@
       <c r="C251" s="5" t="n"/>
       <c r="D251" s="5" t="n"/>
       <c r="E251" s="5" t="n"/>
+      <c r="F251" s="5" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="3" t="n"/>
@@ -2361,6 +2622,7 @@
       <c r="C252" s="5" t="n"/>
       <c r="D252" s="5" t="n"/>
       <c r="E252" s="5" t="n"/>
+      <c r="F252" s="5" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="3" t="n"/>
@@ -2368,6 +2630,7 @@
       <c r="C253" s="5" t="n"/>
       <c r="D253" s="5" t="n"/>
       <c r="E253" s="5" t="n"/>
+      <c r="F253" s="5" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="3" t="n"/>
@@ -2375,6 +2638,7 @@
       <c r="C254" s="5" t="n"/>
       <c r="D254" s="5" t="n"/>
       <c r="E254" s="5" t="n"/>
+      <c r="F254" s="5" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="3" t="n"/>
@@ -2382,6 +2646,7 @@
       <c r="C255" s="5" t="n"/>
       <c r="D255" s="5" t="n"/>
       <c r="E255" s="5" t="n"/>
+      <c r="F255" s="5" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="3" t="n"/>
@@ -2389,6 +2654,7 @@
       <c r="C256" s="5" t="n"/>
       <c r="D256" s="5" t="n"/>
       <c r="E256" s="5" t="n"/>
+      <c r="F256" s="5" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="3" t="n"/>
@@ -2396,6 +2662,7 @@
       <c r="C257" s="5" t="n"/>
       <c r="D257" s="5" t="n"/>
       <c r="E257" s="5" t="n"/>
+      <c r="F257" s="5" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n"/>
@@ -2403,6 +2670,7 @@
       <c r="C258" s="5" t="n"/>
       <c r="D258" s="5" t="n"/>
       <c r="E258" s="5" t="n"/>
+      <c r="F258" s="5" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="3" t="n"/>
@@ -2410,6 +2678,7 @@
       <c r="C259" s="5" t="n"/>
       <c r="D259" s="5" t="n"/>
       <c r="E259" s="5" t="n"/>
+      <c r="F259" s="5" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="3" t="n"/>
@@ -2417,6 +2686,7 @@
       <c r="C260" s="5" t="n"/>
       <c r="D260" s="5" t="n"/>
       <c r="E260" s="5" t="n"/>
+      <c r="F260" s="5" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="3" t="n"/>
@@ -2424,6 +2694,7 @@
       <c r="C261" s="5" t="n"/>
       <c r="D261" s="5" t="n"/>
       <c r="E261" s="5" t="n"/>
+      <c r="F261" s="5" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="3" t="n"/>
@@ -2431,6 +2702,7 @@
       <c r="C262" s="5" t="n"/>
       <c r="D262" s="5" t="n"/>
       <c r="E262" s="5" t="n"/>
+      <c r="F262" s="5" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="3" t="n"/>
@@ -2438,6 +2710,7 @@
       <c r="C263" s="5" t="n"/>
       <c r="D263" s="5" t="n"/>
       <c r="E263" s="5" t="n"/>
+      <c r="F263" s="5" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="3" t="n"/>
@@ -2445,6 +2718,7 @@
       <c r="C264" s="5" t="n"/>
       <c r="D264" s="5" t="n"/>
       <c r="E264" s="5" t="n"/>
+      <c r="F264" s="5" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="3" t="n"/>
@@ -2452,6 +2726,7 @@
       <c r="C265" s="5" t="n"/>
       <c r="D265" s="5" t="n"/>
       <c r="E265" s="5" t="n"/>
+      <c r="F265" s="5" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="3" t="n"/>
@@ -2459,6 +2734,7 @@
       <c r="C266" s="5" t="n"/>
       <c r="D266" s="5" t="n"/>
       <c r="E266" s="5" t="n"/>
+      <c r="F266" s="5" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="3" t="n"/>
@@ -2466,6 +2742,7 @@
       <c r="C267" s="5" t="n"/>
       <c r="D267" s="5" t="n"/>
       <c r="E267" s="5" t="n"/>
+      <c r="F267" s="5" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="3" t="n"/>
@@ -2473,6 +2750,7 @@
       <c r="C268" s="5" t="n"/>
       <c r="D268" s="5" t="n"/>
       <c r="E268" s="5" t="n"/>
+      <c r="F268" s="5" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="3" t="n"/>
@@ -2480,6 +2758,7 @@
       <c r="C269" s="5" t="n"/>
       <c r="D269" s="5" t="n"/>
       <c r="E269" s="5" t="n"/>
+      <c r="F269" s="5" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="3" t="n"/>
@@ -2487,6 +2766,7 @@
       <c r="C270" s="5" t="n"/>
       <c r="D270" s="5" t="n"/>
       <c r="E270" s="5" t="n"/>
+      <c r="F270" s="5" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="3" t="n"/>
@@ -2494,6 +2774,7 @@
       <c r="C271" s="5" t="n"/>
       <c r="D271" s="5" t="n"/>
       <c r="E271" s="5" t="n"/>
+      <c r="F271" s="5" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="3" t="n"/>
@@ -2501,6 +2782,7 @@
       <c r="C272" s="5" t="n"/>
       <c r="D272" s="5" t="n"/>
       <c r="E272" s="5" t="n"/>
+      <c r="F272" s="5" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="3" t="n"/>
@@ -2508,6 +2790,7 @@
       <c r="C273" s="5" t="n"/>
       <c r="D273" s="5" t="n"/>
       <c r="E273" s="5" t="n"/>
+      <c r="F273" s="5" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="3" t="n"/>
@@ -2515,6 +2798,7 @@
       <c r="C274" s="5" t="n"/>
       <c r="D274" s="5" t="n"/>
       <c r="E274" s="5" t="n"/>
+      <c r="F274" s="5" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="3" t="n"/>
@@ -2522,6 +2806,7 @@
       <c r="C275" s="5" t="n"/>
       <c r="D275" s="5" t="n"/>
       <c r="E275" s="5" t="n"/>
+      <c r="F275" s="5" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="3" t="n"/>
@@ -2529,6 +2814,7 @@
       <c r="C276" s="5" t="n"/>
       <c r="D276" s="5" t="n"/>
       <c r="E276" s="5" t="n"/>
+      <c r="F276" s="5" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="3" t="n"/>
@@ -2536,6 +2822,7 @@
       <c r="C277" s="5" t="n"/>
       <c r="D277" s="5" t="n"/>
       <c r="E277" s="5" t="n"/>
+      <c r="F277" s="5" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="3" t="n"/>
@@ -2543,6 +2830,7 @@
       <c r="C278" s="5" t="n"/>
       <c r="D278" s="5" t="n"/>
       <c r="E278" s="5" t="n"/>
+      <c r="F278" s="5" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="3" t="n"/>
@@ -2550,6 +2838,7 @@
       <c r="C279" s="5" t="n"/>
       <c r="D279" s="5" t="n"/>
       <c r="E279" s="5" t="n"/>
+      <c r="F279" s="5" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="3" t="n"/>
@@ -2557,6 +2846,7 @@
       <c r="C280" s="5" t="n"/>
       <c r="D280" s="5" t="n"/>
       <c r="E280" s="5" t="n"/>
+      <c r="F280" s="5" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="3" t="n"/>
@@ -2564,6 +2854,7 @@
       <c r="C281" s="5" t="n"/>
       <c r="D281" s="5" t="n"/>
       <c r="E281" s="5" t="n"/>
+      <c r="F281" s="5" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="3" t="n"/>
@@ -2571,6 +2862,7 @@
       <c r="C282" s="5" t="n"/>
       <c r="D282" s="5" t="n"/>
       <c r="E282" s="5" t="n"/>
+      <c r="F282" s="5" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="3" t="n"/>
@@ -2578,6 +2870,7 @@
       <c r="C283" s="5" t="n"/>
       <c r="D283" s="5" t="n"/>
       <c r="E283" s="5" t="n"/>
+      <c r="F283" s="5" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="3" t="n"/>
@@ -2585,6 +2878,7 @@
       <c r="C284" s="5" t="n"/>
       <c r="D284" s="5" t="n"/>
       <c r="E284" s="5" t="n"/>
+      <c r="F284" s="5" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="3" t="n"/>
@@ -2592,6 +2886,7 @@
       <c r="C285" s="5" t="n"/>
       <c r="D285" s="5" t="n"/>
       <c r="E285" s="5" t="n"/>
+      <c r="F285" s="5" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="3" t="n"/>
@@ -2599,6 +2894,7 @@
       <c r="C286" s="5" t="n"/>
       <c r="D286" s="5" t="n"/>
       <c r="E286" s="5" t="n"/>
+      <c r="F286" s="5" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="3" t="n"/>
@@ -2606,6 +2902,7 @@
       <c r="C287" s="5" t="n"/>
       <c r="D287" s="5" t="n"/>
       <c r="E287" s="5" t="n"/>
+      <c r="F287" s="5" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="3" t="n"/>
@@ -2613,6 +2910,7 @@
       <c r="C288" s="5" t="n"/>
       <c r="D288" s="5" t="n"/>
       <c r="E288" s="5" t="n"/>
+      <c r="F288" s="5" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="3" t="n"/>
@@ -2620,6 +2918,7 @@
       <c r="C289" s="5" t="n"/>
       <c r="D289" s="5" t="n"/>
       <c r="E289" s="5" t="n"/>
+      <c r="F289" s="5" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="3" t="n"/>
@@ -2627,6 +2926,7 @@
       <c r="C290" s="5" t="n"/>
       <c r="D290" s="5" t="n"/>
       <c r="E290" s="5" t="n"/>
+      <c r="F290" s="5" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="3" t="n"/>
@@ -2634,6 +2934,7 @@
       <c r="C291" s="5" t="n"/>
       <c r="D291" s="5" t="n"/>
       <c r="E291" s="5" t="n"/>
+      <c r="F291" s="5" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="3" t="n"/>
@@ -2641,6 +2942,7 @@
       <c r="C292" s="5" t="n"/>
       <c r="D292" s="5" t="n"/>
       <c r="E292" s="5" t="n"/>
+      <c r="F292" s="5" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="3" t="n"/>
@@ -2648,6 +2950,7 @@
       <c r="C293" s="5" t="n"/>
       <c r="D293" s="5" t="n"/>
       <c r="E293" s="5" t="n"/>
+      <c r="F293" s="5" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="3" t="n"/>
@@ -2655,6 +2958,7 @@
       <c r="C294" s="5" t="n"/>
       <c r="D294" s="5" t="n"/>
       <c r="E294" s="5" t="n"/>
+      <c r="F294" s="5" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="3" t="n"/>
@@ -2662,6 +2966,7 @@
       <c r="C295" s="5" t="n"/>
       <c r="D295" s="5" t="n"/>
       <c r="E295" s="5" t="n"/>
+      <c r="F295" s="5" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="3" t="n"/>
@@ -2669,6 +2974,7 @@
       <c r="C296" s="5" t="n"/>
       <c r="D296" s="5" t="n"/>
       <c r="E296" s="5" t="n"/>
+      <c r="F296" s="5" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="3" t="n"/>
@@ -2676,6 +2982,7 @@
       <c r="C297" s="5" t="n"/>
       <c r="D297" s="5" t="n"/>
       <c r="E297" s="5" t="n"/>
+      <c r="F297" s="5" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="3" t="n"/>
@@ -2683,6 +2990,7 @@
       <c r="C298" s="5" t="n"/>
       <c r="D298" s="5" t="n"/>
       <c r="E298" s="5" t="n"/>
+      <c r="F298" s="5" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="3" t="n"/>
@@ -2690,6 +2998,7 @@
       <c r="C299" s="5" t="n"/>
       <c r="D299" s="5" t="n"/>
       <c r="E299" s="5" t="n"/>
+      <c r="F299" s="5" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="3" t="n"/>
@@ -2697,6 +3006,7 @@
       <c r="C300" s="5" t="n"/>
       <c r="D300" s="5" t="n"/>
       <c r="E300" s="5" t="n"/>
+      <c r="F300" s="5" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="3" t="n"/>
@@ -2704,6 +3014,7 @@
       <c r="C301" s="5" t="n"/>
       <c r="D301" s="5" t="n"/>
       <c r="E301" s="5" t="n"/>
+      <c r="F301" s="5" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="3" t="n"/>
@@ -2711,6 +3022,7 @@
       <c r="C302" s="5" t="n"/>
       <c r="D302" s="5" t="n"/>
       <c r="E302" s="5" t="n"/>
+      <c r="F302" s="5" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="3" t="n"/>
@@ -2718,6 +3030,7 @@
       <c r="C303" s="5" t="n"/>
       <c r="D303" s="5" t="n"/>
       <c r="E303" s="5" t="n"/>
+      <c r="F303" s="5" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="3" t="n"/>
@@ -2725,6 +3038,7 @@
       <c r="C304" s="5" t="n"/>
       <c r="D304" s="5" t="n"/>
       <c r="E304" s="5" t="n"/>
+      <c r="F304" s="5" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="3" t="n"/>
@@ -2732,6 +3046,7 @@
       <c r="C305" s="5" t="n"/>
       <c r="D305" s="5" t="n"/>
       <c r="E305" s="5" t="n"/>
+      <c r="F305" s="5" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="3" t="n"/>
@@ -2739,6 +3054,7 @@
       <c r="C306" s="5" t="n"/>
       <c r="D306" s="5" t="n"/>
       <c r="E306" s="5" t="n"/>
+      <c r="F306" s="5" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="3" t="n"/>
@@ -2746,6 +3062,7 @@
       <c r="C307" s="5" t="n"/>
       <c r="D307" s="5" t="n"/>
       <c r="E307" s="5" t="n"/>
+      <c r="F307" s="5" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="3" t="n"/>
@@ -2753,6 +3070,7 @@
       <c r="C308" s="5" t="n"/>
       <c r="D308" s="5" t="n"/>
       <c r="E308" s="5" t="n"/>
+      <c r="F308" s="5" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="3" t="n"/>
@@ -2760,6 +3078,7 @@
       <c r="C309" s="5" t="n"/>
       <c r="D309" s="5" t="n"/>
       <c r="E309" s="5" t="n"/>
+      <c r="F309" s="5" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="3" t="n"/>
@@ -2767,6 +3086,7 @@
       <c r="C310" s="5" t="n"/>
       <c r="D310" s="5" t="n"/>
       <c r="E310" s="5" t="n"/>
+      <c r="F310" s="5" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="3" t="n"/>
@@ -2774,6 +3094,7 @@
       <c r="C311" s="5" t="n"/>
       <c r="D311" s="5" t="n"/>
       <c r="E311" s="5" t="n"/>
+      <c r="F311" s="5" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="3" t="n"/>
@@ -2781,6 +3102,7 @@
       <c r="C312" s="5" t="n"/>
       <c r="D312" s="5" t="n"/>
       <c r="E312" s="5" t="n"/>
+      <c r="F312" s="5" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="3" t="n"/>
@@ -2788,6 +3110,7 @@
       <c r="C313" s="5" t="n"/>
       <c r="D313" s="5" t="n"/>
       <c r="E313" s="5" t="n"/>
+      <c r="F313" s="5" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="3" t="n"/>
@@ -2795,6 +3118,7 @@
       <c r="C314" s="5" t="n"/>
       <c r="D314" s="5" t="n"/>
       <c r="E314" s="5" t="n"/>
+      <c r="F314" s="5" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="3" t="n"/>
@@ -2802,6 +3126,7 @@
       <c r="C315" s="5" t="n"/>
       <c r="D315" s="5" t="n"/>
       <c r="E315" s="5" t="n"/>
+      <c r="F315" s="5" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="3" t="n"/>
@@ -2809,6 +3134,7 @@
       <c r="C316" s="5" t="n"/>
       <c r="D316" s="5" t="n"/>
       <c r="E316" s="5" t="n"/>
+      <c r="F316" s="5" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="3" t="n"/>
@@ -2816,6 +3142,7 @@
       <c r="C317" s="5" t="n"/>
       <c r="D317" s="5" t="n"/>
       <c r="E317" s="5" t="n"/>
+      <c r="F317" s="5" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="3" t="n"/>
@@ -2823,6 +3150,7 @@
       <c r="C318" s="5" t="n"/>
       <c r="D318" s="5" t="n"/>
       <c r="E318" s="5" t="n"/>
+      <c r="F318" s="5" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="3" t="n"/>
@@ -2830,6 +3158,7 @@
       <c r="C319" s="5" t="n"/>
       <c r="D319" s="5" t="n"/>
       <c r="E319" s="5" t="n"/>
+      <c r="F319" s="5" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="3" t="n"/>
@@ -2837,6 +3166,7 @@
       <c r="C320" s="5" t="n"/>
       <c r="D320" s="5" t="n"/>
       <c r="E320" s="5" t="n"/>
+      <c r="F320" s="5" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="3" t="n"/>
@@ -2844,6 +3174,7 @@
       <c r="C321" s="5" t="n"/>
       <c r="D321" s="5" t="n"/>
       <c r="E321" s="5" t="n"/>
+      <c r="F321" s="5" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="3" t="n"/>
@@ -2851,6 +3182,7 @@
       <c r="C322" s="5" t="n"/>
       <c r="D322" s="5" t="n"/>
       <c r="E322" s="5" t="n"/>
+      <c r="F322" s="5" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="3" t="n"/>
@@ -2858,6 +3190,7 @@
       <c r="C323" s="5" t="n"/>
       <c r="D323" s="5" t="n"/>
       <c r="E323" s="5" t="n"/>
+      <c r="F323" s="5" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="3" t="n"/>
@@ -2865,6 +3198,7 @@
       <c r="C324" s="5" t="n"/>
       <c r="D324" s="5" t="n"/>
       <c r="E324" s="5" t="n"/>
+      <c r="F324" s="5" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="3" t="n"/>
@@ -2872,6 +3206,7 @@
       <c r="C325" s="5" t="n"/>
       <c r="D325" s="5" t="n"/>
       <c r="E325" s="5" t="n"/>
+      <c r="F325" s="5" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="3" t="n"/>
@@ -2879,6 +3214,7 @@
       <c r="C326" s="5" t="n"/>
       <c r="D326" s="5" t="n"/>
       <c r="E326" s="5" t="n"/>
+      <c r="F326" s="5" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="3" t="n"/>
@@ -2886,6 +3222,7 @@
       <c r="C327" s="5" t="n"/>
       <c r="D327" s="5" t="n"/>
       <c r="E327" s="5" t="n"/>
+      <c r="F327" s="5" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="3" t="n"/>
@@ -2893,6 +3230,7 @@
       <c r="C328" s="5" t="n"/>
       <c r="D328" s="5" t="n"/>
       <c r="E328" s="5" t="n"/>
+      <c r="F328" s="5" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="3" t="n"/>
@@ -2900,6 +3238,7 @@
       <c r="C329" s="5" t="n"/>
       <c r="D329" s="5" t="n"/>
       <c r="E329" s="5" t="n"/>
+      <c r="F329" s="5" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="3" t="n"/>
@@ -2907,6 +3246,7 @@
       <c r="C330" s="5" t="n"/>
       <c r="D330" s="5" t="n"/>
       <c r="E330" s="5" t="n"/>
+      <c r="F330" s="5" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="3" t="n"/>
@@ -2914,6 +3254,7 @@
       <c r="C331" s="5" t="n"/>
       <c r="D331" s="5" t="n"/>
       <c r="E331" s="5" t="n"/>
+      <c r="F331" s="5" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="3" t="n"/>
@@ -2921,6 +3262,7 @@
       <c r="C332" s="5" t="n"/>
       <c r="D332" s="5" t="n"/>
       <c r="E332" s="5" t="n"/>
+      <c r="F332" s="5" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="3" t="n"/>
@@ -2928,6 +3270,7 @@
       <c r="C333" s="5" t="n"/>
       <c r="D333" s="5" t="n"/>
       <c r="E333" s="5" t="n"/>
+      <c r="F333" s="5" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="3" t="n"/>
@@ -2935,6 +3278,7 @@
       <c r="C334" s="5" t="n"/>
       <c r="D334" s="5" t="n"/>
       <c r="E334" s="5" t="n"/>
+      <c r="F334" s="5" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="3" t="n"/>
@@ -2942,6 +3286,7 @@
       <c r="C335" s="5" t="n"/>
       <c r="D335" s="5" t="n"/>
       <c r="E335" s="5" t="n"/>
+      <c r="F335" s="5" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="3" t="n"/>
@@ -2949,6 +3294,7 @@
       <c r="C336" s="5" t="n"/>
       <c r="D336" s="5" t="n"/>
       <c r="E336" s="5" t="n"/>
+      <c r="F336" s="5" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="3" t="n"/>
@@ -2956,6 +3302,7 @@
       <c r="C337" s="5" t="n"/>
       <c r="D337" s="5" t="n"/>
       <c r="E337" s="5" t="n"/>
+      <c r="F337" s="5" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="3" t="n"/>
@@ -2963,6 +3310,7 @@
       <c r="C338" s="5" t="n"/>
       <c r="D338" s="5" t="n"/>
       <c r="E338" s="5" t="n"/>
+      <c r="F338" s="5" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="3" t="n"/>
@@ -2970,6 +3318,7 @@
       <c r="C339" s="5" t="n"/>
       <c r="D339" s="5" t="n"/>
       <c r="E339" s="5" t="n"/>
+      <c r="F339" s="5" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="3" t="n"/>
@@ -2977,6 +3326,7 @@
       <c r="C340" s="5" t="n"/>
       <c r="D340" s="5" t="n"/>
       <c r="E340" s="5" t="n"/>
+      <c r="F340" s="5" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="3" t="n"/>
@@ -2984,6 +3334,7 @@
       <c r="C341" s="5" t="n"/>
       <c r="D341" s="5" t="n"/>
       <c r="E341" s="5" t="n"/>
+      <c r="F341" s="5" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="3" t="n"/>
@@ -2991,6 +3342,7 @@
       <c r="C342" s="5" t="n"/>
       <c r="D342" s="5" t="n"/>
       <c r="E342" s="5" t="n"/>
+      <c r="F342" s="5" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="3" t="n"/>
@@ -2998,6 +3350,7 @@
       <c r="C343" s="5" t="n"/>
       <c r="D343" s="5" t="n"/>
       <c r="E343" s="5" t="n"/>
+      <c r="F343" s="5" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="3" t="n"/>
@@ -3005,6 +3358,7 @@
       <c r="C344" s="5" t="n"/>
       <c r="D344" s="5" t="n"/>
       <c r="E344" s="5" t="n"/>
+      <c r="F344" s="5" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="3" t="n"/>
@@ -3012,6 +3366,7 @@
       <c r="C345" s="5" t="n"/>
       <c r="D345" s="5" t="n"/>
       <c r="E345" s="5" t="n"/>
+      <c r="F345" s="5" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="3" t="n"/>
@@ -3019,6 +3374,7 @@
       <c r="C346" s="5" t="n"/>
       <c r="D346" s="5" t="n"/>
       <c r="E346" s="5" t="n"/>
+      <c r="F346" s="5" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="3" t="n"/>
@@ -3026,6 +3382,7 @@
       <c r="C347" s="5" t="n"/>
       <c r="D347" s="5" t="n"/>
       <c r="E347" s="5" t="n"/>
+      <c r="F347" s="5" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="3" t="n"/>
@@ -3033,6 +3390,7 @@
       <c r="C348" s="5" t="n"/>
       <c r="D348" s="5" t="n"/>
       <c r="E348" s="5" t="n"/>
+      <c r="F348" s="5" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="3" t="n"/>
@@ -3040,6 +3398,7 @@
       <c r="C349" s="5" t="n"/>
       <c r="D349" s="5" t="n"/>
       <c r="E349" s="5" t="n"/>
+      <c r="F349" s="5" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="3" t="n"/>
@@ -3047,6 +3406,7 @@
       <c r="C350" s="5" t="n"/>
       <c r="D350" s="5" t="n"/>
       <c r="E350" s="5" t="n"/>
+      <c r="F350" s="5" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="3" t="n"/>
@@ -3054,6 +3414,7 @@
       <c r="C351" s="5" t="n"/>
       <c r="D351" s="5" t="n"/>
       <c r="E351" s="5" t="n"/>
+      <c r="F351" s="5" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="3" t="n"/>
@@ -3061,6 +3422,7 @@
       <c r="C352" s="5" t="n"/>
       <c r="D352" s="5" t="n"/>
       <c r="E352" s="5" t="n"/>
+      <c r="F352" s="5" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="3" t="n"/>
@@ -3068,6 +3430,7 @@
       <c r="C353" s="5" t="n"/>
       <c r="D353" s="5" t="n"/>
       <c r="E353" s="5" t="n"/>
+      <c r="F353" s="5" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="3" t="n"/>
@@ -3075,6 +3438,7 @@
       <c r="C354" s="5" t="n"/>
       <c r="D354" s="5" t="n"/>
       <c r="E354" s="5" t="n"/>
+      <c r="F354" s="5" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="3" t="n"/>
@@ -3082,6 +3446,7 @@
       <c r="C355" s="5" t="n"/>
       <c r="D355" s="5" t="n"/>
       <c r="E355" s="5" t="n"/>
+      <c r="F355" s="5" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="3" t="n"/>
@@ -3089,6 +3454,7 @@
       <c r="C356" s="5" t="n"/>
       <c r="D356" s="5" t="n"/>
       <c r="E356" s="5" t="n"/>
+      <c r="F356" s="5" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="3" t="n"/>
@@ -3096,6 +3462,7 @@
       <c r="C357" s="5" t="n"/>
       <c r="D357" s="5" t="n"/>
       <c r="E357" s="5" t="n"/>
+      <c r="F357" s="5" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="3" t="n"/>
@@ -3103,6 +3470,7 @@
       <c r="C358" s="5" t="n"/>
       <c r="D358" s="5" t="n"/>
       <c r="E358" s="5" t="n"/>
+      <c r="F358" s="5" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="3" t="n"/>
@@ -3110,6 +3478,7 @@
       <c r="C359" s="5" t="n"/>
       <c r="D359" s="5" t="n"/>
       <c r="E359" s="5" t="n"/>
+      <c r="F359" s="5" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="3" t="n"/>
@@ -3117,6 +3486,7 @@
       <c r="C360" s="5" t="n"/>
       <c r="D360" s="5" t="n"/>
       <c r="E360" s="5" t="n"/>
+      <c r="F360" s="5" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="3" t="n"/>
@@ -3124,6 +3494,7 @@
       <c r="C361" s="5" t="n"/>
       <c r="D361" s="5" t="n"/>
       <c r="E361" s="5" t="n"/>
+      <c r="F361" s="5" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="3" t="n"/>
@@ -3131,6 +3502,7 @@
       <c r="C362" s="5" t="n"/>
       <c r="D362" s="5" t="n"/>
       <c r="E362" s="5" t="n"/>
+      <c r="F362" s="5" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="3" t="n"/>
@@ -3138,6 +3510,7 @@
       <c r="C363" s="5" t="n"/>
       <c r="D363" s="5" t="n"/>
       <c r="E363" s="5" t="n"/>
+      <c r="F363" s="5" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="3" t="n"/>
@@ -3145,6 +3518,7 @@
       <c r="C364" s="5" t="n"/>
       <c r="D364" s="5" t="n"/>
       <c r="E364" s="5" t="n"/>
+      <c r="F364" s="5" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="3" t="n"/>
@@ -3152,6 +3526,7 @@
       <c r="C365" s="5" t="n"/>
       <c r="D365" s="5" t="n"/>
       <c r="E365" s="5" t="n"/>
+      <c r="F365" s="5" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="3" t="n"/>
@@ -3159,6 +3534,7 @@
       <c r="C366" s="5" t="n"/>
       <c r="D366" s="5" t="n"/>
       <c r="E366" s="5" t="n"/>
+      <c r="F366" s="5" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="3" t="n"/>
@@ -3166,6 +3542,7 @@
       <c r="C367" s="5" t="n"/>
       <c r="D367" s="5" t="n"/>
       <c r="E367" s="5" t="n"/>
+      <c r="F367" s="5" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="3" t="n"/>
@@ -3173,6 +3550,7 @@
       <c r="C368" s="5" t="n"/>
       <c r="D368" s="5" t="n"/>
       <c r="E368" s="5" t="n"/>
+      <c r="F368" s="5" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="3" t="n"/>
@@ -3180,6 +3558,7 @@
       <c r="C369" s="5" t="n"/>
       <c r="D369" s="5" t="n"/>
       <c r="E369" s="5" t="n"/>
+      <c r="F369" s="5" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="3" t="n"/>
@@ -3187,6 +3566,7 @@
       <c r="C370" s="5" t="n"/>
       <c r="D370" s="5" t="n"/>
       <c r="E370" s="5" t="n"/>
+      <c r="F370" s="5" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="3" t="n"/>
@@ -3194,6 +3574,7 @@
       <c r="C371" s="5" t="n"/>
       <c r="D371" s="5" t="n"/>
       <c r="E371" s="5" t="n"/>
+      <c r="F371" s="5" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="3" t="n"/>
@@ -3201,6 +3582,7 @@
       <c r="C372" s="5" t="n"/>
       <c r="D372" s="5" t="n"/>
       <c r="E372" s="5" t="n"/>
+      <c r="F372" s="5" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="3" t="n"/>
@@ -3208,6 +3590,7 @@
       <c r="C373" s="5" t="n"/>
       <c r="D373" s="5" t="n"/>
       <c r="E373" s="5" t="n"/>
+      <c r="F373" s="5" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="3" t="n"/>
@@ -3215,6 +3598,7 @@
       <c r="C374" s="5" t="n"/>
       <c r="D374" s="5" t="n"/>
       <c r="E374" s="5" t="n"/>
+      <c r="F374" s="5" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="3" t="n"/>
@@ -3222,6 +3606,7 @@
       <c r="C375" s="5" t="n"/>
       <c r="D375" s="5" t="n"/>
       <c r="E375" s="5" t="n"/>
+      <c r="F375" s="5" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="3" t="n"/>
@@ -3229,6 +3614,7 @@
       <c r="C376" s="5" t="n"/>
       <c r="D376" s="5" t="n"/>
       <c r="E376" s="5" t="n"/>
+      <c r="F376" s="5" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="3" t="n"/>
@@ -3236,6 +3622,7 @@
       <c r="C377" s="5" t="n"/>
       <c r="D377" s="5" t="n"/>
       <c r="E377" s="5" t="n"/>
+      <c r="F377" s="5" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="3" t="n"/>
@@ -3243,6 +3630,7 @@
       <c r="C378" s="5" t="n"/>
       <c r="D378" s="5" t="n"/>
       <c r="E378" s="5" t="n"/>
+      <c r="F378" s="5" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="3" t="n"/>
@@ -3250,6 +3638,7 @@
       <c r="C379" s="5" t="n"/>
       <c r="D379" s="5" t="n"/>
       <c r="E379" s="5" t="n"/>
+      <c r="F379" s="5" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="3" t="n"/>
@@ -3257,6 +3646,7 @@
       <c r="C380" s="5" t="n"/>
       <c r="D380" s="5" t="n"/>
       <c r="E380" s="5" t="n"/>
+      <c r="F380" s="5" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="3" t="n"/>
@@ -3264,6 +3654,7 @@
       <c r="C381" s="5" t="n"/>
       <c r="D381" s="5" t="n"/>
       <c r="E381" s="5" t="n"/>
+      <c r="F381" s="5" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="3" t="n"/>
@@ -3271,6 +3662,7 @@
       <c r="C382" s="5" t="n"/>
       <c r="D382" s="5" t="n"/>
       <c r="E382" s="5" t="n"/>
+      <c r="F382" s="5" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="3" t="n"/>
@@ -3278,6 +3670,7 @@
       <c r="C383" s="5" t="n"/>
       <c r="D383" s="5" t="n"/>
       <c r="E383" s="5" t="n"/>
+      <c r="F383" s="5" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="3" t="n"/>
@@ -3285,6 +3678,7 @@
       <c r="C384" s="5" t="n"/>
       <c r="D384" s="5" t="n"/>
       <c r="E384" s="5" t="n"/>
+      <c r="F384" s="5" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="3" t="n"/>
@@ -3292,6 +3686,7 @@
       <c r="C385" s="5" t="n"/>
       <c r="D385" s="5" t="n"/>
       <c r="E385" s="5" t="n"/>
+      <c r="F385" s="5" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="3" t="n"/>
@@ -3299,6 +3694,7 @@
       <c r="C386" s="5" t="n"/>
       <c r="D386" s="5" t="n"/>
       <c r="E386" s="5" t="n"/>
+      <c r="F386" s="5" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="3" t="n"/>
@@ -3306,6 +3702,7 @@
       <c r="C387" s="5" t="n"/>
       <c r="D387" s="5" t="n"/>
       <c r="E387" s="5" t="n"/>
+      <c r="F387" s="5" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="3" t="n"/>
@@ -3313,6 +3710,7 @@
       <c r="C388" s="5" t="n"/>
       <c r="D388" s="5" t="n"/>
       <c r="E388" s="5" t="n"/>
+      <c r="F388" s="5" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="3" t="n"/>
@@ -3320,6 +3718,7 @@
       <c r="C389" s="5" t="n"/>
       <c r="D389" s="5" t="n"/>
       <c r="E389" s="5" t="n"/>
+      <c r="F389" s="5" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="3" t="n"/>
@@ -3327,6 +3726,7 @@
       <c r="C390" s="5" t="n"/>
       <c r="D390" s="5" t="n"/>
       <c r="E390" s="5" t="n"/>
+      <c r="F390" s="5" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="3" t="n"/>
@@ -3334,6 +3734,7 @@
       <c r="C391" s="5" t="n"/>
       <c r="D391" s="5" t="n"/>
       <c r="E391" s="5" t="n"/>
+      <c r="F391" s="5" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="3" t="n"/>
@@ -3341,6 +3742,7 @@
       <c r="C392" s="5" t="n"/>
       <c r="D392" s="5" t="n"/>
       <c r="E392" s="5" t="n"/>
+      <c r="F392" s="5" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="3" t="n"/>
@@ -3348,6 +3750,7 @@
       <c r="C393" s="5" t="n"/>
       <c r="D393" s="5" t="n"/>
       <c r="E393" s="5" t="n"/>
+      <c r="F393" s="5" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="3" t="n"/>
@@ -3355,6 +3758,7 @@
       <c r="C394" s="5" t="n"/>
       <c r="D394" s="5" t="n"/>
       <c r="E394" s="5" t="n"/>
+      <c r="F394" s="5" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="3" t="n"/>
@@ -3362,6 +3766,7 @@
       <c r="C395" s="5" t="n"/>
       <c r="D395" s="5" t="n"/>
       <c r="E395" s="5" t="n"/>
+      <c r="F395" s="5" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="3" t="n"/>
@@ -3369,6 +3774,7 @@
       <c r="C396" s="5" t="n"/>
       <c r="D396" s="5" t="n"/>
       <c r="E396" s="5" t="n"/>
+      <c r="F396" s="5" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="3" t="n"/>
@@ -3376,6 +3782,7 @@
       <c r="C397" s="5" t="n"/>
       <c r="D397" s="5" t="n"/>
       <c r="E397" s="5" t="n"/>
+      <c r="F397" s="5" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="3" t="n"/>
@@ -3383,6 +3790,7 @@
       <c r="C398" s="5" t="n"/>
       <c r="D398" s="5" t="n"/>
       <c r="E398" s="5" t="n"/>
+      <c r="F398" s="5" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="3" t="n"/>
@@ -3390,6 +3798,7 @@
       <c r="C399" s="5" t="n"/>
       <c r="D399" s="5" t="n"/>
       <c r="E399" s="5" t="n"/>
+      <c r="F399" s="5" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="3" t="n"/>
@@ -3397,6 +3806,7 @@
       <c r="C400" s="5" t="n"/>
       <c r="D400" s="5" t="n"/>
       <c r="E400" s="5" t="n"/>
+      <c r="F400" s="5" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="3" t="n"/>
@@ -3404,6 +3814,7 @@
       <c r="C401" s="5" t="n"/>
       <c r="D401" s="5" t="n"/>
       <c r="E401" s="5" t="n"/>
+      <c r="F401" s="5" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="3" t="n"/>
@@ -3411,6 +3822,7 @@
       <c r="C402" s="5" t="n"/>
       <c r="D402" s="5" t="n"/>
       <c r="E402" s="5" t="n"/>
+      <c r="F402" s="5" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="3" t="n"/>
@@ -3418,6 +3830,7 @@
       <c r="C403" s="5" t="n"/>
       <c r="D403" s="5" t="n"/>
       <c r="E403" s="5" t="n"/>
+      <c r="F403" s="5" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="3" t="n"/>
@@ -3425,6 +3838,7 @@
       <c r="C404" s="5" t="n"/>
       <c r="D404" s="5" t="n"/>
       <c r="E404" s="5" t="n"/>
+      <c r="F404" s="5" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="3" t="n"/>
@@ -3432,6 +3846,7 @@
       <c r="C405" s="5" t="n"/>
       <c r="D405" s="5" t="n"/>
       <c r="E405" s="5" t="n"/>
+      <c r="F405" s="5" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="3" t="n"/>
@@ -3439,6 +3854,7 @@
       <c r="C406" s="5" t="n"/>
       <c r="D406" s="5" t="n"/>
       <c r="E406" s="5" t="n"/>
+      <c r="F406" s="5" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="3" t="n"/>
@@ -3446,6 +3862,7 @@
       <c r="C407" s="5" t="n"/>
       <c r="D407" s="5" t="n"/>
       <c r="E407" s="5" t="n"/>
+      <c r="F407" s="5" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="3" t="n"/>
@@ -3453,6 +3870,7 @@
       <c r="C408" s="5" t="n"/>
       <c r="D408" s="5" t="n"/>
       <c r="E408" s="5" t="n"/>
+      <c r="F408" s="5" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="3" t="n"/>
@@ -3460,6 +3878,7 @@
       <c r="C409" s="5" t="n"/>
       <c r="D409" s="5" t="n"/>
       <c r="E409" s="5" t="n"/>
+      <c r="F409" s="5" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="3" t="n"/>
@@ -3467,6 +3886,7 @@
       <c r="C410" s="5" t="n"/>
       <c r="D410" s="5" t="n"/>
       <c r="E410" s="5" t="n"/>
+      <c r="F410" s="5" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="3" t="n"/>
@@ -3474,6 +3894,7 @@
       <c r="C411" s="5" t="n"/>
       <c r="D411" s="5" t="n"/>
       <c r="E411" s="5" t="n"/>
+      <c r="F411" s="5" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="3" t="n"/>
@@ -3481,6 +3902,7 @@
       <c r="C412" s="5" t="n"/>
       <c r="D412" s="5" t="n"/>
       <c r="E412" s="5" t="n"/>
+      <c r="F412" s="5" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="3" t="n"/>
@@ -3488,6 +3910,7 @@
       <c r="C413" s="5" t="n"/>
       <c r="D413" s="5" t="n"/>
       <c r="E413" s="5" t="n"/>
+      <c r="F413" s="5" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="3" t="n"/>
@@ -3495,6 +3918,7 @@
       <c r="C414" s="5" t="n"/>
       <c r="D414" s="5" t="n"/>
       <c r="E414" s="5" t="n"/>
+      <c r="F414" s="5" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="3" t="n"/>
@@ -3502,6 +3926,7 @@
       <c r="C415" s="5" t="n"/>
       <c r="D415" s="5" t="n"/>
       <c r="E415" s="5" t="n"/>
+      <c r="F415" s="5" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="3" t="n"/>
@@ -3509,6 +3934,7 @@
       <c r="C416" s="5" t="n"/>
       <c r="D416" s="5" t="n"/>
       <c r="E416" s="5" t="n"/>
+      <c r="F416" s="5" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="3" t="n"/>
@@ -3516,6 +3942,7 @@
       <c r="C417" s="5" t="n"/>
       <c r="D417" s="5" t="n"/>
       <c r="E417" s="5" t="n"/>
+      <c r="F417" s="5" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="3" t="n"/>
@@ -3523,6 +3950,7 @@
       <c r="C418" s="5" t="n"/>
       <c r="D418" s="5" t="n"/>
       <c r="E418" s="5" t="n"/>
+      <c r="F418" s="5" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="3" t="n"/>
@@ -3530,6 +3958,7 @@
       <c r="C419" s="5" t="n"/>
       <c r="D419" s="5" t="n"/>
       <c r="E419" s="5" t="n"/>
+      <c r="F419" s="5" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="3" t="n"/>
@@ -3537,6 +3966,7 @@
       <c r="C420" s="5" t="n"/>
       <c r="D420" s="5" t="n"/>
       <c r="E420" s="5" t="n"/>
+      <c r="F420" s="5" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="3" t="n"/>
@@ -3544,6 +3974,7 @@
       <c r="C421" s="5" t="n"/>
       <c r="D421" s="5" t="n"/>
       <c r="E421" s="5" t="n"/>
+      <c r="F421" s="5" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="3" t="n"/>
@@ -3551,6 +3982,7 @@
       <c r="C422" s="5" t="n"/>
       <c r="D422" s="5" t="n"/>
       <c r="E422" s="5" t="n"/>
+      <c r="F422" s="5" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="3" t="n"/>
@@ -3558,6 +3990,7 @@
       <c r="C423" s="5" t="n"/>
       <c r="D423" s="5" t="n"/>
       <c r="E423" s="5" t="n"/>
+      <c r="F423" s="5" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="3" t="n"/>
@@ -3565,6 +3998,7 @@
       <c r="C424" s="5" t="n"/>
       <c r="D424" s="5" t="n"/>
       <c r="E424" s="5" t="n"/>
+      <c r="F424" s="5" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="3" t="n"/>
@@ -3572,6 +4006,7 @@
       <c r="C425" s="5" t="n"/>
       <c r="D425" s="5" t="n"/>
       <c r="E425" s="5" t="n"/>
+      <c r="F425" s="5" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="3" t="n"/>
@@ -3579,6 +4014,7 @@
       <c r="C426" s="5" t="n"/>
       <c r="D426" s="5" t="n"/>
       <c r="E426" s="5" t="n"/>
+      <c r="F426" s="5" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="3" t="n"/>
@@ -3586,6 +4022,7 @@
       <c r="C427" s="5" t="n"/>
       <c r="D427" s="5" t="n"/>
       <c r="E427" s="5" t="n"/>
+      <c r="F427" s="5" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="3" t="n"/>
@@ -3593,6 +4030,7 @@
       <c r="C428" s="5" t="n"/>
       <c r="D428" s="5" t="n"/>
       <c r="E428" s="5" t="n"/>
+      <c r="F428" s="5" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="3" t="n"/>
@@ -3600,6 +4038,7 @@
       <c r="C429" s="5" t="n"/>
       <c r="D429" s="5" t="n"/>
       <c r="E429" s="5" t="n"/>
+      <c r="F429" s="5" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="3" t="n"/>
@@ -3607,6 +4046,7 @@
       <c r="C430" s="5" t="n"/>
       <c r="D430" s="5" t="n"/>
       <c r="E430" s="5" t="n"/>
+      <c r="F430" s="5" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="3" t="n"/>
@@ -3614,6 +4054,7 @@
       <c r="C431" s="5" t="n"/>
       <c r="D431" s="5" t="n"/>
       <c r="E431" s="5" t="n"/>
+      <c r="F431" s="5" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="3" t="n"/>
@@ -3621,6 +4062,7 @@
       <c r="C432" s="5" t="n"/>
       <c r="D432" s="5" t="n"/>
       <c r="E432" s="5" t="n"/>
+      <c r="F432" s="5" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="3" t="n"/>
@@ -3628,6 +4070,7 @@
       <c r="C433" s="5" t="n"/>
       <c r="D433" s="5" t="n"/>
       <c r="E433" s="5" t="n"/>
+      <c r="F433" s="5" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="3" t="n"/>
@@ -3635,6 +4078,7 @@
       <c r="C434" s="5" t="n"/>
       <c r="D434" s="5" t="n"/>
       <c r="E434" s="5" t="n"/>
+      <c r="F434" s="5" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="3" t="n"/>
@@ -3642,6 +4086,7 @@
       <c r="C435" s="5" t="n"/>
       <c r="D435" s="5" t="n"/>
       <c r="E435" s="5" t="n"/>
+      <c r="F435" s="5" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="3" t="n"/>
@@ -3649,6 +4094,7 @@
       <c r="C436" s="5" t="n"/>
       <c r="D436" s="5" t="n"/>
       <c r="E436" s="5" t="n"/>
+      <c r="F436" s="5" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="3" t="n"/>
@@ -3656,6 +4102,7 @@
       <c r="C437" s="5" t="n"/>
       <c r="D437" s="5" t="n"/>
       <c r="E437" s="5" t="n"/>
+      <c r="F437" s="5" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="3" t="n"/>
@@ -3663,6 +4110,7 @@
       <c r="C438" s="5" t="n"/>
       <c r="D438" s="5" t="n"/>
       <c r="E438" s="5" t="n"/>
+      <c r="F438" s="5" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="3" t="n"/>
@@ -3670,6 +4118,7 @@
       <c r="C439" s="5" t="n"/>
       <c r="D439" s="5" t="n"/>
       <c r="E439" s="5" t="n"/>
+      <c r="F439" s="5" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="3" t="n"/>
@@ -3677,6 +4126,7 @@
       <c r="C440" s="5" t="n"/>
       <c r="D440" s="5" t="n"/>
       <c r="E440" s="5" t="n"/>
+      <c r="F440" s="5" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="3" t="n"/>
@@ -3684,6 +4134,7 @@
       <c r="C441" s="5" t="n"/>
       <c r="D441" s="5" t="n"/>
       <c r="E441" s="5" t="n"/>
+      <c r="F441" s="5" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="3" t="n"/>
@@ -3691,6 +4142,7 @@
       <c r="C442" s="5" t="n"/>
       <c r="D442" s="5" t="n"/>
       <c r="E442" s="5" t="n"/>
+      <c r="F442" s="5" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="3" t="n"/>
@@ -3698,6 +4150,7 @@
       <c r="C443" s="5" t="n"/>
       <c r="D443" s="5" t="n"/>
       <c r="E443" s="5" t="n"/>
+      <c r="F443" s="5" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="3" t="n"/>
@@ -3705,6 +4158,7 @@
       <c r="C444" s="5" t="n"/>
       <c r="D444" s="5" t="n"/>
       <c r="E444" s="5" t="n"/>
+      <c r="F444" s="5" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="3" t="n"/>
@@ -3712,6 +4166,7 @@
       <c r="C445" s="5" t="n"/>
       <c r="D445" s="5" t="n"/>
       <c r="E445" s="5" t="n"/>
+      <c r="F445" s="5" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="3" t="n"/>
@@ -3719,6 +4174,7 @@
       <c r="C446" s="5" t="n"/>
       <c r="D446" s="5" t="n"/>
       <c r="E446" s="5" t="n"/>
+      <c r="F446" s="5" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="3" t="n"/>
@@ -3726,6 +4182,7 @@
       <c r="C447" s="5" t="n"/>
       <c r="D447" s="5" t="n"/>
       <c r="E447" s="5" t="n"/>
+      <c r="F447" s="5" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="3" t="n"/>
@@ -3733,6 +4190,7 @@
       <c r="C448" s="5" t="n"/>
       <c r="D448" s="5" t="n"/>
       <c r="E448" s="5" t="n"/>
+      <c r="F448" s="5" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="3" t="n"/>
@@ -3740,6 +4198,7 @@
       <c r="C449" s="5" t="n"/>
       <c r="D449" s="5" t="n"/>
       <c r="E449" s="5" t="n"/>
+      <c r="F449" s="5" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="3" t="n"/>
@@ -3747,6 +4206,7 @@
       <c r="C450" s="5" t="n"/>
       <c r="D450" s="5" t="n"/>
       <c r="E450" s="5" t="n"/>
+      <c r="F450" s="5" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="3" t="n"/>
@@ -3754,6 +4214,7 @@
       <c r="C451" s="5" t="n"/>
       <c r="D451" s="5" t="n"/>
       <c r="E451" s="5" t="n"/>
+      <c r="F451" s="5" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="3" t="n"/>
@@ -3761,6 +4222,7 @@
       <c r="C452" s="5" t="n"/>
       <c r="D452" s="5" t="n"/>
       <c r="E452" s="5" t="n"/>
+      <c r="F452" s="5" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="3" t="n"/>
@@ -3768,6 +4230,7 @@
       <c r="C453" s="5" t="n"/>
       <c r="D453" s="5" t="n"/>
       <c r="E453" s="5" t="n"/>
+      <c r="F453" s="5" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="3" t="n"/>
@@ -3775,6 +4238,7 @@
       <c r="C454" s="5" t="n"/>
       <c r="D454" s="5" t="n"/>
       <c r="E454" s="5" t="n"/>
+      <c r="F454" s="5" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="3" t="n"/>
@@ -3782,6 +4246,7 @@
       <c r="C455" s="5" t="n"/>
       <c r="D455" s="5" t="n"/>
       <c r="E455" s="5" t="n"/>
+      <c r="F455" s="5" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="3" t="n"/>
@@ -3789,6 +4254,7 @@
       <c r="C456" s="5" t="n"/>
       <c r="D456" s="5" t="n"/>
       <c r="E456" s="5" t="n"/>
+      <c r="F456" s="5" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="3" t="n"/>
@@ -3796,6 +4262,7 @@
       <c r="C457" s="5" t="n"/>
       <c r="D457" s="5" t="n"/>
       <c r="E457" s="5" t="n"/>
+      <c r="F457" s="5" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="3" t="n"/>
@@ -3803,6 +4270,7 @@
       <c r="C458" s="5" t="n"/>
       <c r="D458" s="5" t="n"/>
       <c r="E458" s="5" t="n"/>
+      <c r="F458" s="5" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="3" t="n"/>
@@ -3810,6 +4278,7 @@
       <c r="C459" s="5" t="n"/>
       <c r="D459" s="5" t="n"/>
       <c r="E459" s="5" t="n"/>
+      <c r="F459" s="5" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="3" t="n"/>
@@ -3817,6 +4286,7 @@
       <c r="C460" s="5" t="n"/>
       <c r="D460" s="5" t="n"/>
       <c r="E460" s="5" t="n"/>
+      <c r="F460" s="5" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="3" t="n"/>
@@ -3824,6 +4294,7 @@
       <c r="C461" s="5" t="n"/>
       <c r="D461" s="5" t="n"/>
       <c r="E461" s="5" t="n"/>
+      <c r="F461" s="5" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="3" t="n"/>
@@ -3831,6 +4302,7 @@
       <c r="C462" s="5" t="n"/>
       <c r="D462" s="5" t="n"/>
       <c r="E462" s="5" t="n"/>
+      <c r="F462" s="5" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="3" t="n"/>
@@ -3838,6 +4310,7 @@
       <c r="C463" s="5" t="n"/>
       <c r="D463" s="5" t="n"/>
       <c r="E463" s="5" t="n"/>
+      <c r="F463" s="5" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="3" t="n"/>
@@ -3845,6 +4318,7 @@
       <c r="C464" s="5" t="n"/>
       <c r="D464" s="5" t="n"/>
       <c r="E464" s="5" t="n"/>
+      <c r="F464" s="5" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="3" t="n"/>
@@ -3852,6 +4326,7 @@
       <c r="C465" s="5" t="n"/>
       <c r="D465" s="5" t="n"/>
       <c r="E465" s="5" t="n"/>
+      <c r="F465" s="5" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="3" t="n"/>
@@ -3859,6 +4334,7 @@
       <c r="C466" s="5" t="n"/>
       <c r="D466" s="5" t="n"/>
       <c r="E466" s="5" t="n"/>
+      <c r="F466" s="5" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="3" t="n"/>
@@ -3866,6 +4342,7 @@
       <c r="C467" s="5" t="n"/>
       <c r="D467" s="5" t="n"/>
       <c r="E467" s="5" t="n"/>
+      <c r="F467" s="5" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="3" t="n"/>
@@ -3873,6 +4350,7 @@
       <c r="C468" s="5" t="n"/>
       <c r="D468" s="5" t="n"/>
       <c r="E468" s="5" t="n"/>
+      <c r="F468" s="5" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="3" t="n"/>
@@ -3880,6 +4358,7 @@
       <c r="C469" s="5" t="n"/>
       <c r="D469" s="5" t="n"/>
       <c r="E469" s="5" t="n"/>
+      <c r="F469" s="5" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="3" t="n"/>
@@ -3887,6 +4366,7 @@
       <c r="C470" s="5" t="n"/>
       <c r="D470" s="5" t="n"/>
       <c r="E470" s="5" t="n"/>
+      <c r="F470" s="5" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="3" t="n"/>
@@ -3894,6 +4374,7 @@
       <c r="C471" s="5" t="n"/>
       <c r="D471" s="5" t="n"/>
       <c r="E471" s="5" t="n"/>
+      <c r="F471" s="5" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="3" t="n"/>
@@ -3901,6 +4382,7 @@
       <c r="C472" s="5" t="n"/>
       <c r="D472" s="5" t="n"/>
       <c r="E472" s="5" t="n"/>
+      <c r="F472" s="5" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="3" t="n"/>
@@ -3908,6 +4390,7 @@
       <c r="C473" s="5" t="n"/>
       <c r="D473" s="5" t="n"/>
       <c r="E473" s="5" t="n"/>
+      <c r="F473" s="5" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="3" t="n"/>
@@ -3915,6 +4398,7 @@
       <c r="C474" s="5" t="n"/>
       <c r="D474" s="5" t="n"/>
       <c r="E474" s="5" t="n"/>
+      <c r="F474" s="5" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="3" t="n"/>
@@ -3922,6 +4406,7 @@
       <c r="C475" s="5" t="n"/>
       <c r="D475" s="5" t="n"/>
       <c r="E475" s="5" t="n"/>
+      <c r="F475" s="5" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="3" t="n"/>
@@ -3929,6 +4414,7 @@
       <c r="C476" s="5" t="n"/>
       <c r="D476" s="5" t="n"/>
       <c r="E476" s="5" t="n"/>
+      <c r="F476" s="5" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="3" t="n"/>
@@ -3936,6 +4422,7 @@
       <c r="C477" s="5" t="n"/>
       <c r="D477" s="5" t="n"/>
       <c r="E477" s="5" t="n"/>
+      <c r="F477" s="5" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="3" t="n"/>
@@ -3943,6 +4430,7 @@
       <c r="C478" s="5" t="n"/>
       <c r="D478" s="5" t="n"/>
       <c r="E478" s="5" t="n"/>
+      <c r="F478" s="5" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="3" t="n"/>
@@ -3950,6 +4438,7 @@
       <c r="C479" s="5" t="n"/>
       <c r="D479" s="5" t="n"/>
       <c r="E479" s="5" t="n"/>
+      <c r="F479" s="5" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="3" t="n"/>
@@ -3957,6 +4446,7 @@
       <c r="C480" s="5" t="n"/>
       <c r="D480" s="5" t="n"/>
       <c r="E480" s="5" t="n"/>
+      <c r="F480" s="5" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="3" t="n"/>
@@ -3964,6 +4454,7 @@
       <c r="C481" s="5" t="n"/>
       <c r="D481" s="5" t="n"/>
       <c r="E481" s="5" t="n"/>
+      <c r="F481" s="5" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="3" t="n"/>
@@ -3971,6 +4462,7 @@
       <c r="C482" s="5" t="n"/>
       <c r="D482" s="5" t="n"/>
       <c r="E482" s="5" t="n"/>
+      <c r="F482" s="5" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="3" t="n"/>
@@ -3978,6 +4470,7 @@
       <c r="C483" s="5" t="n"/>
       <c r="D483" s="5" t="n"/>
       <c r="E483" s="5" t="n"/>
+      <c r="F483" s="5" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="3" t="n"/>
@@ -3985,6 +4478,7 @@
       <c r="C484" s="5" t="n"/>
       <c r="D484" s="5" t="n"/>
       <c r="E484" s="5" t="n"/>
+      <c r="F484" s="5" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="3" t="n"/>
@@ -3992,6 +4486,7 @@
       <c r="C485" s="5" t="n"/>
       <c r="D485" s="5" t="n"/>
       <c r="E485" s="5" t="n"/>
+      <c r="F485" s="5" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="3" t="n"/>
@@ -3999,6 +4494,7 @@
       <c r="C486" s="5" t="n"/>
       <c r="D486" s="5" t="n"/>
       <c r="E486" s="5" t="n"/>
+      <c r="F486" s="5" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="3" t="n"/>
@@ -4006,6 +4502,7 @@
       <c r="C487" s="5" t="n"/>
       <c r="D487" s="5" t="n"/>
       <c r="E487" s="5" t="n"/>
+      <c r="F487" s="5" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="3" t="n"/>
@@ -4013,6 +4510,7 @@
       <c r="C488" s="5" t="n"/>
       <c r="D488" s="5" t="n"/>
       <c r="E488" s="5" t="n"/>
+      <c r="F488" s="5" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="3" t="n"/>
@@ -4020,6 +4518,7 @@
       <c r="C489" s="5" t="n"/>
       <c r="D489" s="5" t="n"/>
       <c r="E489" s="5" t="n"/>
+      <c r="F489" s="5" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="3" t="n"/>
@@ -4027,6 +4526,7 @@
       <c r="C490" s="5" t="n"/>
       <c r="D490" s="5" t="n"/>
       <c r="E490" s="5" t="n"/>
+      <c r="F490" s="5" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="3" t="n"/>
@@ -4034,6 +4534,7 @@
       <c r="C491" s="5" t="n"/>
       <c r="D491" s="5" t="n"/>
       <c r="E491" s="5" t="n"/>
+      <c r="F491" s="5" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="3" t="n"/>
@@ -4041,6 +4542,7 @@
       <c r="C492" s="5" t="n"/>
       <c r="D492" s="5" t="n"/>
       <c r="E492" s="5" t="n"/>
+      <c r="F492" s="5" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="3" t="n"/>
@@ -4048,6 +4550,7 @@
       <c r="C493" s="5" t="n"/>
       <c r="D493" s="5" t="n"/>
       <c r="E493" s="5" t="n"/>
+      <c r="F493" s="5" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="3" t="n"/>
@@ -4055,6 +4558,7 @@
       <c r="C494" s="5" t="n"/>
       <c r="D494" s="5" t="n"/>
       <c r="E494" s="5" t="n"/>
+      <c r="F494" s="5" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="3" t="n"/>
@@ -4062,6 +4566,7 @@
       <c r="C495" s="5" t="n"/>
       <c r="D495" s="5" t="n"/>
       <c r="E495" s="5" t="n"/>
+      <c r="F495" s="5" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="3" t="n"/>
@@ -4069,6 +4574,7 @@
       <c r="C496" s="5" t="n"/>
       <c r="D496" s="5" t="n"/>
       <c r="E496" s="5" t="n"/>
+      <c r="F496" s="5" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="3" t="n"/>
@@ -4076,6 +4582,7 @@
       <c r="C497" s="5" t="n"/>
       <c r="D497" s="5" t="n"/>
       <c r="E497" s="5" t="n"/>
+      <c r="F497" s="5" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="3" t="n"/>
@@ -4083,6 +4590,7 @@
       <c r="C498" s="5" t="n"/>
       <c r="D498" s="5" t="n"/>
       <c r="E498" s="5" t="n"/>
+      <c r="F498" s="5" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="3" t="n"/>
@@ -4090,6 +4598,7 @@
       <c r="C499" s="5" t="n"/>
       <c r="D499" s="5" t="n"/>
       <c r="E499" s="5" t="n"/>
+      <c r="F499" s="5" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="3" t="n"/>
@@ -4097,6 +4606,7 @@
       <c r="C500" s="5" t="n"/>
       <c r="D500" s="5" t="n"/>
       <c r="E500" s="5" t="n"/>
+      <c r="F500" s="5" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="3" t="n"/>
@@ -4104,9 +4614,10 @@
       <c r="C501" s="5" t="n"/>
       <c r="D501" s="5" t="n"/>
       <c r="E501" s="5" t="n"/>
+      <c r="F501" s="5" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Nom" error="Le nom doit faire entre 2 et 80 caractères." type="textLength" errorStyle="warning" operator="between">
       <formula1>2</formula1>
       <formula2>80</formula2>
@@ -4122,6 +4633,9 @@
     </dataValidation>
     <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Stock" error="Écrivez un nombre entier (0 ou plus)." type="whole" errorStyle="warning" operator="greaterThanOrEqual">
       <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Prix de gros" error="Écrivez un nombre entier supérieur à 0, sans « F », ou laissez la case vide." type="whole" errorStyle="warning" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4417,7 +4931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:C26"/>
+  <dimension ref="B1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4561,91 +5075,103 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="B16" s="8" t="inlineStr">
+    <row r="15" ht="48" customHeight="1">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Prix de gros</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Facultatif. Le prix que vous appliquez quand vous livrez chez un client ou un revendeur. Au comptoir, c’est toujours le prix de vente. Case vide : le prix de vente s’applique aussi aux livraisons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Si une ligne est refusée</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>nom manquant ou trop court</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>La colonne Nom est vide ou fait moins de 2 caractères.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="B18" s="9" t="inlineStr">
         <is>
+          <t>nom manquant ou trop court</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>La colonne Nom est vide ou fait moins de 2 caractères.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
           <t>prix de vente manquant ou invalide</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>Le prix de vente est vide, à 0, ou n’est pas un nombre.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="B19" s="9" t="inlineStr">
+    <row r="20" ht="34" customHeight="1">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>ce produit existe déjà</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Le produit est déjà dans votre carte, ou en double dans le fichier. Un produit existant n’est jamais écrasé.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="B20" s="9" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>accents abîmés</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Si « Bière » apparaît « Bi?re », enregistrez de nouveau en « CSV UTF-8 ».</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="B22" s="8" t="inlineStr">
+    <row r="23" ht="24" customHeight="1">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Bon à savoir</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>• Ne changez pas les titres des colonnes de la feuille « Mes produits », et gardez-la en première position.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>• Les exemples de la feuille « Exemples » ne sont pas importés : copiez-les dans « Mes produits » si vous voulez vous en servir.</t>
+          <t>• Ne changez pas les titres des colonnes de la feuille « Mes produits », et gardez-la en première position.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>• Vous pouvez importer plusieurs fois : les produits déjà présents sont simplement refusés.</t>
+          <t>• Les exemples de la feuille « Exemples » ne sont pas importés : copiez-les dans « Mes produits » si vous voulez vous en servir.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>• Vous pouvez importer plusieurs fois : les produits déjà présents sont simplement refusés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>• Une question ? WhatsApp 05 65 75 03 03, ou mondje.ci/modeles.</t>
         </is>
@@ -4655,12 +5181,12 @@
   <mergeCells count="10">
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B1:C1"/>
   </mergeCells>
@@ -4675,7 +5201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4683,6 +5209,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4702,6 +5229,7 @@
       <c r="C3" s="15" t="n"/>
       <c r="D3" s="15" t="n"/>
       <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -4727,6 +5255,11 @@
       <c r="E4" s="16" t="inlineStr">
         <is>
           <t>Stock</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>Prix de gros</t>
         </is>
       </c>
     </row>
@@ -4824,6 +5357,7 @@
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -4849,6 +5383,11 @@
       <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Stock</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Prix de gros</t>
         </is>
       </c>
     </row>
@@ -4946,6 +5485,7 @@
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -4973,6 +5513,11 @@
           <t>Stock</t>
         </is>
       </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Prix de gros</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
@@ -5060,7 +5605,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>